<commit_message>
feat(F-NAR-009): ramifiées COL-031 et COL-032
Ouvertures monde d’abord (radiateur, presse-agrumes). Audio plus tard.
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-031.xlsx
+++ b/stories/arbres/TREE-COL-031.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -552,7 +552,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Barnabé attend puis parle</t>
+          <t>Les moufles et le bateau en papier</t>
         </is>
       </c>
     </row>
@@ -843,6 +843,18 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>voix-roles-v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fil_rouge</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Les moufles sèchent sur le radiateur. Un bateau en papier attend sur le rebord. Victorino lève la main, il attend, puis il parle, avec papa et maman.</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1197,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Barnabé arrive en classe avec maman. Il lève la main. Il faut attendre. Puis il pourra parler.</t>
+          <t>Le radiateur fait tic, tout petit. Les moufles bleues sèchent dessus. Elles sentent encore la pluie. La vitre de la classe est embuée. Un bateau en papier attend sur le rebord. Dehors, la gouttière chante. Ça sent l'orange, dans la poche. Papa a glissé le fruit, ce matin. L'orange est pour plus tard, Victorino. Le manteau goutte encore, au portemanteau. Tu as les pieds au sec ? Oui, maman. Le lino a un carré de lumière. Un crayon bleu a roulé près d'une table. Tu lèves la main, d'accord ? D'accord, papa. On peut attendre. Puis on parle. En ce moment, Victorino entre dans la classe. Le tapis est gris, un peu rêche. La table sent le bois. La fenêtre tremble un peu, sous la pluie. J'ai une chose à dire. Moi aussi. On peut attendre d'abord. Victorino lève la main. Il attend. Le bateau en papier ne bouge pas.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1325,10 +1337,41 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé arrive en classe avec maman. Il lève la main. Il faut attendre. Puis il pourra parler.</t>
-        </is>
-      </c>
-      <c r="AX2" t="inlineStr"/>
+          <t>narrateur|Le radiateur fait tic, tout petit.
+narrateur|Les moufles bleues sèchent dessus.
+narrateur|Elles sentent encore la pluie.
+narrateur|La vitre de la classe est embuée.
+narrateur|Un bateau en papier attend sur le rebord.
+narrateur|Dehors, la gouttière chante.
+narrateur|Ça sent l'orange, dans la poche.
+narrateur|Papa a glissé le fruit, ce matin.
+papa|L'orange est pour plus tard, Victorino.
+maman|Le manteau goutte encore, au portemanteau.
+maman|Tu as les pieds au sec ?
+enfant-m|Oui, maman.
+narrateur|Le lino a un carré de lumière.
+narrateur|Un crayon bleu a roulé près d'une table.
+papa|Tu lèves la main, d'accord ?
+enfant-m|D'accord, papa.
+maman|On peut attendre.
+maman|Puis on parle.
+narrateur|En ce moment, Victorino entre dans la classe.
+narrateur|Le tapis est gris, un peu rêche.
+narrateur|La table sent le bois.
+narrateur|La fenêtre tremble un peu, sous la pluie.
+enfant-m|J'ai une chose à dire.
+papa|Moi aussi.
+papa|On peut attendre d'abord.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+narrateur|Le bateau en papier ne bouge pas.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>pluie,radiateur</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1353,7 +1396,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre le tapis, la table, ou la fenêtre.</t>
+          <t>Dans la classe, trois endroits attendent. Le tapis, la table, ou la fenêtre ? On lève la main. On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1517,7 +1560,11 @@
       <c r="AV3" s="2" t="inlineStr"/>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre le tapis, la table, ou la fenêtre.</t>
+          <t>narrateur|Dans la classe, trois endroits attendent.
+maman|Le tapis, la table, ou la fenêtre ?
+papa|On lève la main.
+papa|On peut attendre.
+papa|Puis on parle.</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr"/>
@@ -1545,7 +1592,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sur le tapis, Barnabé lève la main. Il attend. Puis il parle.</t>
+          <t>Victorino pose un genou sur le tapis. Le tapis est gris, un peu rêche. Un bouton bleu s'est perdu dans les poils. Le radiateur chauffe encore, tout près. Moi, je raconte le bouton d'abord. Maman parle jusqu'au bout. Victorino a une chose à dire. Il lève la main. Il attend. Le bouton est tout rond. Oui. C'est ton tour. Tu as attendu. On lève la main. On peut attendre. Puis on parle. Victorino touche le bouton, tout doux. Le tapis chatouille encore le genou.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1685,7 +1732,24 @@
       <c r="AV4" s="2" t="inlineStr"/>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sur le tapis, Barnabé lève la main. Il attend. Puis il parle.</t>
+          <t>narrateur|Victorino pose un genou sur le tapis.
+narrateur|Le tapis est gris, un peu rêche.
+narrateur|Un bouton bleu s'est perdu dans les poils.
+narrateur|Le radiateur chauffe encore, tout près.
+maman|Moi, je raconte le bouton d'abord.
+narrateur|Maman parle jusqu'au bout.
+narrateur|Victorino a une chose à dire.
+narrateur|Il lève la main.
+narrateur|Il attend.
+enfant-m|Le bouton est tout rond.
+papa|Oui.
+papa|C'est ton tour.
+papa|Tu as attendu.
+maman|On lève la main.
+maman|On peut attendre.
+maman|Puis on parle.
+narrateur|Victorino touche le bouton, tout doux.
+narrateur|Le tapis chatouille encore le genou.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr"/>
@@ -1713,7 +1777,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sur le tapis, que fait Barnabé d'abord ?</t>
+          <t>Sur le tapis, Victorino veut parler. Que fait-il d'abord ?</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1869,7 +1933,8 @@
       </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Sur le tapis, que fait Barnabé d'abord ?</t>
+          <t>narrateur|Sur le tapis, Victorino veut parler.
+maman|Que fait-il d'abord ?</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr"/>
@@ -1897,7 +1962,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Barnabé a attendu. Puis il a parlé.</t>
+          <t>Oui. On lève la main. On peut attendre. Puis on parle. Victorino souffle un peu. Sa main redescend, tout doux. J'ai attendu. Bravo. C'est du bon travail. Le bouton bleu reste dans les poils.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2041,7 +2106,16 @@
       </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé a attendu. Puis il a parlé.</t>
+          <t>maman|Oui.
+maman|On lève la main.
+maman|On peut attendre.
+maman|Puis on parle.
+narrateur|Victorino souffle un peu.
+narrateur|Sa main redescend, tout doux.
+enfant-m|J'ai attendu.
+papa|Bravo.
+papa|C'est du bon travail.
+narrateur|Le bouton bleu reste dans les poils.</t>
         </is>
       </c>
       <c r="AX6" t="inlineStr"/>
@@ -2069,7 +2143,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre l'histoire, la chanson, ou le dessin.</t>
+          <t>Trois choses attendent, dans la classe. L'histoire, la chanson, ou le dessin ? On lève la main. On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -2233,7 +2307,11 @@
       <c r="AV7" s="2" t="inlineStr"/>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre l'histoire, la chanson, ou le dessin.</t>
+          <t>narrateur|Trois choses attendent, dans la classe.
+maman|L'histoire, la chanson, ou le dessin ?
+papa|On lève la main.
+papa|On peut attendre.
+papa|Puis on parle.</t>
         </is>
       </c>
       <c r="AX7" t="inlineStr"/>
@@ -2261,7 +2339,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Barnabé attend. Puis il parle.</t>
+          <t>Maman ouvre un livre d'images. Une page sent le papier, un peu sec. Un bateau y flotte, tout blanc. Moi, je lis l'histoire d'abord. Maman lit jusqu'au bout. Victorino lève la main. Il attend. Le bateau a une voile. Oui. C'est ton tour. On peut attendre. Puis on parle. Victorino touche le papier, tout léger. Bravo. Tu as attendu. Le livre repose sur le tapis gris. On est encore sur le tapis. On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -2401,10 +2479,32 @@
       <c r="AV8" s="2" t="inlineStr"/>
       <c r="AW8" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé attend. Puis il parle.</t>
-        </is>
-      </c>
-      <c r="AX8" t="inlineStr"/>
+          <t>narrateur|Maman ouvre un livre d'images.
+narrateur|Une page sent le papier, un peu sec.
+narrateur|Un bateau y flotte, tout blanc.
+maman|Moi, je lis l'histoire d'abord.
+narrateur|Maman lit jusqu'au bout.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Le bateau a une voile.
+papa|Oui.
+papa|C'est ton tour.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino touche le papier, tout léger.
+maman|Bravo.
+maman|Tu as attendu.
+narrateur|Le livre repose sur le tapis gris.
+narrateur|On est encore sur le tapis.
+maman|On peut attendre.
+maman|Puis on parle.</t>
+        </is>
+      </c>
+      <c r="AX8" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2429,7 +2529,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre Léa, Tom, ou Sami.</t>
+          <t>Trois objets sont là, tout près. Le doudou, le camion, ou le gobelet ? On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -2597,7 +2697,10 @@
       </c>
       <c r="AW9" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre Léa, Tom, ou Sami.</t>
+          <t>narrateur|Trois objets sont là, tout près.
+papa|Le doudou, le camion, ou le gobelet ?
+maman|On peut attendre.
+maman|Puis on parle.</t>
         </is>
       </c>
       <c r="AX9" t="inlineStr"/>
@@ -2625,7 +2728,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Léa. Il a attendu. Puis il a parlé, à le tapis, pendant l'histoire.</t>
+          <t>Le doudou est gris, un peu râpé. Une oreille est encore chaude. Il sent l'orange, tout doux. Victorino a encore le doudou, sur le tapis. Le doudou écoute le livre, sur le tapis. C'était l'histoire. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le doudou reste sur le tapis.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -2765,7 +2868,22 @@
       <c r="AV10" s="2" t="inlineStr"/>
       <c r="AW10" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Léa. Il a attendu. Puis il a parlé, à le tapis, pendant l'histoire.</t>
+          <t>narrateur|Le doudou est gris, un peu râpé.
+narrateur|Une oreille est encore chaude.
+narrateur|Il sent l'orange, tout doux.
+narrateur|Victorino a encore le doudou, sur le tapis.
+narrateur|Le doudou écoute le livre, sur le tapis.
+narrateur|C'était l'histoire.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le doudou reste sur le tapis.</t>
         </is>
       </c>
       <c r="AX10" t="inlineStr"/>
@@ -2793,7 +2911,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi le tapis, l'histoire, et le doudou. Bravo, Victorino. C'est du bon travail. Le doudou garde l'oreille chaude, tout calme. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -2933,7 +3051,14 @@
       <c r="AV11" s="2" t="inlineStr"/>
       <c r="AW11" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi le tapis, l'histoire, et le doudou.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|Le doudou garde l'oreille chaude, tout calme.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX11" t="inlineStr"/>
@@ -2961,7 +3086,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Tom. Il a attendu. Puis il a parlé, à le tapis, pendant l'histoire.</t>
+          <t>Le camion est rouge, tout petit. Une roue crisse, tout fin. Une goutte de pluie brille sur le toit. Victorino a encore le camion, sur le tapis. Le camion se gare près du livre. C'était l'histoire. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le camion reste sur le tapis.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -3101,10 +3226,29 @@
       <c r="AV12" s="2" t="inlineStr"/>
       <c r="AW12" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Tom. Il a attendu. Puis il a parlé, à le tapis, pendant l'histoire.</t>
-        </is>
-      </c>
-      <c r="AX12" t="inlineStr"/>
+          <t>narrateur|Le camion est rouge, tout petit.
+narrateur|Une roue crisse, tout fin.
+narrateur|Une goutte de pluie brille sur le toit.
+narrateur|Victorino a encore le camion, sur le tapis.
+narrateur|Le camion se gare près du livre.
+narrateur|C'était l'histoire.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le camion reste sur le tapis.</t>
+        </is>
+      </c>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>camion</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3129,7 +3273,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi le tapis, l'histoire, et le camion. Bravo, Victorino. C'est du bon travail. Le camion s'endort, une roue encore tiède. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -3269,7 +3413,14 @@
       <c r="AV13" s="2" t="inlineStr"/>
       <c r="AW13" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi le tapis, l'histoire, et le camion.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|Le camion s'endort, une roue encore tiède.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX13" t="inlineStr"/>
@@ -3297,7 +3448,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Sami. Il a attendu. Puis il a parlé, à le tapis, pendant l'histoire.</t>
+          <t>Le gobelet est jaune, un peu froid. L'eau tremble au fond, tout calme. Un reflet de fenêtre y danse. Victorino a encore le gobelet, sur le tapis. Le gobelet jaunit une page, tout doux. C'était l'histoire. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le gobelet reste sur le tapis.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -3437,7 +3588,22 @@
       <c r="AV14" s="2" t="inlineStr"/>
       <c r="AW14" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Sami. Il a attendu. Puis il a parlé, à le tapis, pendant l'histoire.</t>
+          <t>narrateur|Le gobelet est jaune, un peu froid.
+narrateur|L'eau tremble au fond, tout calme.
+narrateur|Un reflet de fenêtre y danse.
+narrateur|Victorino a encore le gobelet, sur le tapis.
+narrateur|Le gobelet jaunit une page, tout doux.
+narrateur|C'était l'histoire.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le gobelet reste sur le tapis.</t>
         </is>
       </c>
       <c r="AX14" t="inlineStr"/>
@@ -3465,7 +3631,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi le tapis, l'histoire, et le gobelet. Bravo, Victorino. C'est du bon travail. L'eau du gobelet ne tremble plus. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -3605,7 +3771,14 @@
       <c r="AV15" s="2" t="inlineStr"/>
       <c r="AW15" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi le tapis, l'histoire, et le gobelet.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|L'eau du gobelet ne tremble plus.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX15" t="inlineStr"/>
@@ -3633,7 +3806,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Barnabé attend. Puis il parle.</t>
+          <t>Papa tapote la table, tout doux. Ça fait un petit toc, comme la pluie. Moi, je chante la gouttière d'abord. Papa chante jusqu'au bout. Victorino lève la main. Il attend. Je peux chanter ? Oui. Tu as attendu. Puis on parle. Victorino chante tout bas, une petite pluie. Bravo, Victorino. On lève la main, même pour chanter. Les moufles bleues bougent un peu, au radiateur. Le tapis étouffe un peu le toc de papa. On est encore sur le tapis. On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -3773,7 +3946,24 @@
       <c r="AV16" s="2" t="inlineStr"/>
       <c r="AW16" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé attend. Puis il parle.</t>
+          <t>narrateur|Papa tapote la table, tout doux.
+narrateur|Ça fait un petit toc, comme la pluie.
+papa|Moi, je chante la gouttière d'abord.
+narrateur|Papa chante jusqu'au bout.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Je peux chanter ?
+maman|Oui.
+maman|Tu as attendu.
+maman|Puis on parle.
+narrateur|Victorino chante tout bas, une petite pluie.
+papa|Bravo, Victorino.
+papa|On lève la main, même pour chanter.
+narrateur|Les moufles bleues bougent un peu, au radiateur.
+narrateur|Le tapis étouffe un peu le toc de papa.
+narrateur|On est encore sur le tapis.
+maman|On peut attendre.
+maman|Puis on parle.</t>
         </is>
       </c>
       <c r="AX16" t="inlineStr"/>
@@ -3801,7 +3991,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre Léa, Tom, ou Sami.</t>
+          <t>Trois objets sont là, tout près. Le doudou, le camion, ou le gobelet ? On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -3969,7 +4159,10 @@
       </c>
       <c r="AW17" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre Léa, Tom, ou Sami.</t>
+          <t>narrateur|Trois objets sont là, tout près.
+papa|Le doudou, le camion, ou le gobelet ?
+maman|On peut attendre.
+maman|Puis on parle.</t>
         </is>
       </c>
       <c r="AX17" t="inlineStr"/>
@@ -3997,7 +4190,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Léa. Il a attendu. Puis il a parlé, à le tapis, pendant la chanson.</t>
+          <t>Le doudou est gris, un peu râpé. Une oreille est encore chaude. Il sent l'orange, tout doux. Victorino a encore le doudou, sur le tapis. Le doudou se berce, avec la chanson. C'était la chanson. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le doudou reste sur le tapis.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -4137,7 +4330,22 @@
       <c r="AV18" s="2" t="inlineStr"/>
       <c r="AW18" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Léa. Il a attendu. Puis il a parlé, à le tapis, pendant la chanson.</t>
+          <t>narrateur|Le doudou est gris, un peu râpé.
+narrateur|Une oreille est encore chaude.
+narrateur|Il sent l'orange, tout doux.
+narrateur|Victorino a encore le doudou, sur le tapis.
+narrateur|Le doudou se berce, avec la chanson.
+narrateur|C'était la chanson.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le doudou reste sur le tapis.</t>
         </is>
       </c>
       <c r="AX18" t="inlineStr"/>
@@ -4165,7 +4373,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi le tapis, la chanson, et le doudou. Bravo, Victorino. C'est du bon travail. Le doudou garde l'oreille chaude, tout calme. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -4305,7 +4513,14 @@
       <c r="AV19" s="2" t="inlineStr"/>
       <c r="AW19" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi le tapis, la chanson, et le doudou.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|Le doudou garde l'oreille chaude, tout calme.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX19" t="inlineStr"/>
@@ -4333,7 +4548,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Tom. Il a attendu. Puis il a parlé, à le tapis, pendant la chanson.</t>
+          <t>Le camion est rouge, tout petit. Une roue crisse, tout fin. Une goutte de pluie brille sur le toit. Victorino a encore le camion, sur le tapis. La roue du camion crisse, en rythme. C'était la chanson. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le camion reste sur le tapis.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -4473,10 +4688,29 @@
       <c r="AV20" s="2" t="inlineStr"/>
       <c r="AW20" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Tom. Il a attendu. Puis il a parlé, à le tapis, pendant la chanson.</t>
-        </is>
-      </c>
-      <c r="AX20" t="inlineStr"/>
+          <t>narrateur|Le camion est rouge, tout petit.
+narrateur|Une roue crisse, tout fin.
+narrateur|Une goutte de pluie brille sur le toit.
+narrateur|Victorino a encore le camion, sur le tapis.
+narrateur|La roue du camion crisse, en rythme.
+narrateur|C'était la chanson.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le camion reste sur le tapis.</t>
+        </is>
+      </c>
+      <c r="AX20" t="inlineStr">
+        <is>
+          <t>camion</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -4501,7 +4735,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi le tapis, la chanson, et le camion. Bravo, Victorino. C'est du bon travail. Le camion s'endort, une roue encore tiède. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -4641,7 +4875,14 @@
       <c r="AV21" s="2" t="inlineStr"/>
       <c r="AW21" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi le tapis, la chanson, et le camion.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|Le camion s'endort, une roue encore tiède.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX21" t="inlineStr"/>
@@ -4669,7 +4910,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Sami. Il a attendu. Puis il a parlé, à le tapis, pendant la chanson.</t>
+          <t>Le gobelet est jaune, un peu froid. L'eau tremble au fond, tout calme. Un reflet de fenêtre y danse. Victorino a encore le gobelet, sur le tapis. L'eau du gobelet tremble, avec le toc. C'était la chanson. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le gobelet reste sur le tapis.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -4809,7 +5050,22 @@
       <c r="AV22" s="2" t="inlineStr"/>
       <c r="AW22" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Sami. Il a attendu. Puis il a parlé, à le tapis, pendant la chanson.</t>
+          <t>narrateur|Le gobelet est jaune, un peu froid.
+narrateur|L'eau tremble au fond, tout calme.
+narrateur|Un reflet de fenêtre y danse.
+narrateur|Victorino a encore le gobelet, sur le tapis.
+narrateur|L'eau du gobelet tremble, avec le toc.
+narrateur|C'était la chanson.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le gobelet reste sur le tapis.</t>
         </is>
       </c>
       <c r="AX22" t="inlineStr"/>
@@ -4837,7 +5093,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi le tapis, la chanson, et le gobelet. Bravo, Victorino. C'est du bon travail. L'eau du gobelet ne tremble plus. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -4977,7 +5233,14 @@
       <c r="AV23" s="2" t="inlineStr"/>
       <c r="AW23" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi le tapis, la chanson, et le gobelet.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|L'eau du gobelet ne tremble plus.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX23" t="inlineStr"/>
@@ -5005,7 +5268,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Barnabé attend. Puis il parle.</t>
+          <t>Un papier blanc attend, tout lisse. Le crayon bleu a encore sa mine cassée. Moi, je dessine le bateau d'abord. Maman trace une voile, tout lentement. Victorino lève la main. Il attend. Je peux un trait ? Oui. C'est ton tour. On peut attendre. Puis on parle. Victorino pose un trait bleu, tout court. Bravo. Tu as levé la main. Le papier blanc plisse, sur le tapis. On est encore sur le tapis. On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -5145,10 +5408,31 @@
       <c r="AV24" s="2" t="inlineStr"/>
       <c r="AW24" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé attend. Puis il parle.</t>
-        </is>
-      </c>
-      <c r="AX24" t="inlineStr"/>
+          <t>narrateur|Un papier blanc attend, tout lisse.
+narrateur|Le crayon bleu a encore sa mine cassée.
+maman|Moi, je dessine le bateau d'abord.
+narrateur|Maman trace une voile, tout lentement.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Je peux un trait ?
+papa|Oui.
+papa|C'est ton tour.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino pose un trait bleu, tout court.
+maman|Bravo.
+maman|Tu as levé la main.
+narrateur|Le papier blanc plisse, sur le tapis.
+narrateur|On est encore sur le tapis.
+maman|On peut attendre.
+maman|Puis on parle.</t>
+        </is>
+      </c>
+      <c r="AX24" t="inlineStr">
+        <is>
+          <t>crayon</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -5173,7 +5457,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre Léa, Tom, ou Sami.</t>
+          <t>Trois objets sont là, tout près. Le doudou, le camion, ou le gobelet ? On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -5341,7 +5625,10 @@
       </c>
       <c r="AW25" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre Léa, Tom, ou Sami.</t>
+          <t>narrateur|Trois objets sont là, tout près.
+papa|Le doudou, le camion, ou le gobelet ?
+maman|On peut attendre.
+maman|Puis on parle.</t>
         </is>
       </c>
       <c r="AX25" t="inlineStr"/>
@@ -5369,7 +5656,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Léa. Il a attendu. Puis il a parlé, à le tapis, pendant le dessin.</t>
+          <t>Le doudou est gris, un peu râpé. Une oreille est encore chaude. Il sent l'orange, tout doux. Victorino a encore le doudou, sur le tapis. Le doudou pose l'oreille sur le papier. C'était le dessin. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le doudou reste sur le tapis.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -5509,7 +5796,22 @@
       <c r="AV26" s="2" t="inlineStr"/>
       <c r="AW26" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Léa. Il a attendu. Puis il a parlé, à le tapis, pendant le dessin.</t>
+          <t>narrateur|Le doudou est gris, un peu râpé.
+narrateur|Une oreille est encore chaude.
+narrateur|Il sent l'orange, tout doux.
+narrateur|Victorino a encore le doudou, sur le tapis.
+narrateur|Le doudou pose l'oreille sur le papier.
+narrateur|C'était le dessin.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le doudou reste sur le tapis.</t>
         </is>
       </c>
       <c r="AX26" t="inlineStr"/>
@@ -5537,7 +5839,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi le tapis, le dessin, et le doudou. Bravo, Victorino. C'est du bon travail. Le doudou garde l'oreille chaude, tout calme. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -5677,7 +5979,14 @@
       <c r="AV27" s="2" t="inlineStr"/>
       <c r="AW27" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi le tapis, le dessin, et le doudou.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|Le doudou garde l'oreille chaude, tout calme.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX27" t="inlineStr"/>
@@ -5705,7 +6014,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Tom. Il a attendu. Puis il a parlé, à le tapis, pendant le dessin.</t>
+          <t>Le camion est rouge, tout petit. Une roue crisse, tout fin. Une goutte de pluie brille sur le toit. Victorino a encore le camion, sur le tapis. Le camion roule le long du trait bleu. C'était le dessin. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le camion reste sur le tapis.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -5845,10 +6154,29 @@
       <c r="AV28" s="2" t="inlineStr"/>
       <c r="AW28" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Tom. Il a attendu. Puis il a parlé, à le tapis, pendant le dessin.</t>
-        </is>
-      </c>
-      <c r="AX28" t="inlineStr"/>
+          <t>narrateur|Le camion est rouge, tout petit.
+narrateur|Une roue crisse, tout fin.
+narrateur|Une goutte de pluie brille sur le toit.
+narrateur|Victorino a encore le camion, sur le tapis.
+narrateur|Le camion roule le long du trait bleu.
+narrateur|C'était le dessin.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le camion reste sur le tapis.</t>
+        </is>
+      </c>
+      <c r="AX28" t="inlineStr">
+        <is>
+          <t>camion</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -5873,7 +6201,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi le tapis, le dessin, et le camion. Bravo, Victorino. C'est du bon travail. Le camion s'endort, une roue encore tiède. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -6013,7 +6341,14 @@
       <c r="AV29" s="2" t="inlineStr"/>
       <c r="AW29" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi le tapis, le dessin, et le camion.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|Le camion s'endort, une roue encore tiède.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX29" t="inlineStr"/>
@@ -6041,7 +6376,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Sami. Il a attendu. Puis il a parlé, à le tapis, pendant le dessin.</t>
+          <t>Le gobelet est jaune, un peu froid. L'eau tremble au fond, tout calme. Un reflet de fenêtre y danse. Victorino a encore le gobelet, sur le tapis. Une goutte du gobelet manque le papier. C'était le dessin. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le gobelet reste sur le tapis.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -6181,7 +6516,22 @@
       <c r="AV30" s="2" t="inlineStr"/>
       <c r="AW30" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Sami. Il a attendu. Puis il a parlé, à le tapis, pendant le dessin.</t>
+          <t>narrateur|Le gobelet est jaune, un peu froid.
+narrateur|L'eau tremble au fond, tout calme.
+narrateur|Un reflet de fenêtre y danse.
+narrateur|Victorino a encore le gobelet, sur le tapis.
+narrateur|Une goutte du gobelet manque le papier.
+narrateur|C'était le dessin.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le gobelet reste sur le tapis.</t>
         </is>
       </c>
       <c r="AX30" t="inlineStr"/>
@@ -6209,7 +6559,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi le tapis, le dessin, et le gobelet. Bravo, Victorino. C'est du bon travail. L'eau du gobelet ne tremble plus. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -6349,7 +6699,14 @@
       <c r="AV31" s="2" t="inlineStr"/>
       <c r="AW31" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi le tapis, le dessin, et le gobelet.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|L'eau du gobelet ne tremble plus.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX31" t="inlineStr"/>
@@ -6377,7 +6734,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>À la table, Barnabé lève la main. Il attend. Puis il parle.</t>
+          <t>Victorino s'assoit à la table. Le bois sent l'orange, un peu. Un crayon bleu a roulé, tout seul. Une petite tache luisante reste sur le bois. Moi, je raconte le crayon. Papa parle, tout calme. Victorino lève la main. Il attend. Le crayon a une mine cassée. Oui. Merci d'avoir attendu. On peut attendre. Puis on parle. Victorino pose un doigt sur la tache. Elle est un peu collante. Bravo, Victorino. Tu as levé la main.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -6517,7 +6874,23 @@
       <c r="AV32" s="2" t="inlineStr"/>
       <c r="AW32" t="inlineStr">
         <is>
-          <t>narrateur|À la table, Barnabé lève la main. Il attend. Puis il parle.</t>
+          <t>narrateur|Victorino s'assoit à la table.
+narrateur|Le bois sent l'orange, un peu.
+narrateur|Un crayon bleu a roulé, tout seul.
+narrateur|Une petite tache luisante reste sur le bois.
+papa|Moi, je raconte le crayon.
+narrateur|Papa parle, tout calme.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Le crayon a une mine cassée.
+maman|Oui.
+maman|Merci d'avoir attendu.
+maman|On peut attendre.
+maman|Puis on parle.
+narrateur|Victorino pose un doigt sur la tache.
+narrateur|Elle est un peu collante.
+papa|Bravo, Victorino.
+papa|Tu as levé la main.</t>
         </is>
       </c>
       <c r="AX32" t="inlineStr"/>
@@ -6545,7 +6918,7 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>À la table, que fait Barnabé d'abord ?</t>
+          <t>À la table, Victorino lève la main. Et après, on peut attendre ?</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -6701,7 +7074,8 @@
       </c>
       <c r="AW33" t="inlineStr">
         <is>
-          <t>narrateur|À la table, que fait Barnabé d'abord ?</t>
+          <t>narrateur|À la table, Victorino lève la main.
+papa|Et après, on peut attendre ?</t>
         </is>
       </c>
       <c r="AX33" t="inlineStr"/>
@@ -6729,7 +7103,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Oui. Attendre, puis parler.</t>
+          <t>Oui. On peut attendre. Puis on parle. Victorino pose le crayon, tout droit. J'attends mon tour. Bravo, Victorino. La table est à toi, et le tour aussi. La petite tache brille encore.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -6873,7 +7247,14 @@
       </c>
       <c r="AW34" t="inlineStr">
         <is>
-          <t>narrateur|Oui. Attendre, puis parler.</t>
+          <t>papa|Oui.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino pose le crayon, tout droit.
+enfant-m|J'attends mon tour.
+maman|Bravo, Victorino.
+maman|La table est à toi, et le tour aussi.
+narrateur|La petite tache brille encore.</t>
         </is>
       </c>
       <c r="AX34" t="inlineStr"/>
@@ -6901,7 +7282,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre l'histoire, la chanson, ou le dessin.</t>
+          <t>Trois choses attendent, dans la classe. L'histoire, la chanson, ou le dessin ? On lève la main. On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -7065,7 +7446,11 @@
       <c r="AV35" s="2" t="inlineStr"/>
       <c r="AW35" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre l'histoire, la chanson, ou le dessin.</t>
+          <t>narrateur|Trois choses attendent, dans la classe.
+maman|L'histoire, la chanson, ou le dessin ?
+papa|On lève la main.
+papa|On peut attendre.
+papa|Puis on parle.</t>
         </is>
       </c>
       <c r="AX35" t="inlineStr"/>
@@ -7093,7 +7478,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Barnabé attend. Puis il parle.</t>
+          <t>Maman ouvre un livre d'images. Une page sent le papier, un peu sec. Un bateau y flotte, tout blanc. Moi, je lis l'histoire d'abord. Maman lit jusqu'au bout. Victorino lève la main. Il attend. Le bateau a une voile. Oui. C'est ton tour. On peut attendre. Puis on parle. Victorino touche le papier, tout léger. Bravo. Tu as attendu. Le livre glisse un peu, sur le bois. On est encore à la table. On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -7233,10 +7618,32 @@
       <c r="AV36" s="2" t="inlineStr"/>
       <c r="AW36" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé attend. Puis il parle.</t>
-        </is>
-      </c>
-      <c r="AX36" t="inlineStr"/>
+          <t>narrateur|Maman ouvre un livre d'images.
+narrateur|Une page sent le papier, un peu sec.
+narrateur|Un bateau y flotte, tout blanc.
+maman|Moi, je lis l'histoire d'abord.
+narrateur|Maman lit jusqu'au bout.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Le bateau a une voile.
+papa|Oui.
+papa|C'est ton tour.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino touche le papier, tout léger.
+maman|Bravo.
+maman|Tu as attendu.
+narrateur|Le livre glisse un peu, sur le bois.
+narrateur|On est encore à la table.
+maman|On peut attendre.
+maman|Puis on parle.</t>
+        </is>
+      </c>
+      <c r="AX36" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -7261,7 +7668,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre Léa, Tom, ou Sami.</t>
+          <t>Trois objets sont là, tout près. Le doudou, le camion, ou le gobelet ? On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -7429,7 +7836,10 @@
       </c>
       <c r="AW37" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre Léa, Tom, ou Sami.</t>
+          <t>narrateur|Trois objets sont là, tout près.
+papa|Le doudou, le camion, ou le gobelet ?
+maman|On peut attendre.
+maman|Puis on parle.</t>
         </is>
       </c>
       <c r="AX37" t="inlineStr"/>
@@ -7457,7 +7867,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Léa. Il a attendu. Puis il a parlé, à la table, pendant l'histoire.</t>
+          <t>Le doudou est gris, un peu râpé. Une oreille est encore chaude. Il sent l'orange, tout doux. Victorino a encore le doudou, à la table. Le doudou s'assoit contre le livre, à table. C'était l'histoire. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le doudou reste à la table.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -7597,7 +8007,22 @@
       <c r="AV38" s="2" t="inlineStr"/>
       <c r="AW38" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Léa. Il a attendu. Puis il a parlé, à la table, pendant l'histoire.</t>
+          <t>narrateur|Le doudou est gris, un peu râpé.
+narrateur|Une oreille est encore chaude.
+narrateur|Il sent l'orange, tout doux.
+narrateur|Victorino a encore le doudou, à la table.
+narrateur|Le doudou s'assoit contre le livre, à table.
+narrateur|C'était l'histoire.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le doudou reste à la table.</t>
         </is>
       </c>
       <c r="AX38" t="inlineStr"/>
@@ -7625,7 +8050,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi la table, l'histoire, et le doudou. Bravo, Victorino. C'est du bon travail. Le doudou garde l'oreille chaude, tout calme. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -7765,7 +8190,14 @@
       <c r="AV39" s="2" t="inlineStr"/>
       <c r="AW39" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi la table, l'histoire, et le doudou.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|Le doudou garde l'oreille chaude, tout calme.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX39" t="inlineStr"/>
@@ -7793,7 +8225,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Tom. Il a attendu. Puis il a parlé, à la table, pendant l'histoire.</t>
+          <t>Le camion est rouge, tout petit. Une roue crisse, tout fin. Une goutte de pluie brille sur le toit. Victorino a encore le camion, à la table. Le camion attend au bord du bois. C'était l'histoire. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le camion reste à la table.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -7933,10 +8365,29 @@
       <c r="AV40" s="2" t="inlineStr"/>
       <c r="AW40" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Tom. Il a attendu. Puis il a parlé, à la table, pendant l'histoire.</t>
-        </is>
-      </c>
-      <c r="AX40" t="inlineStr"/>
+          <t>narrateur|Le camion est rouge, tout petit.
+narrateur|Une roue crisse, tout fin.
+narrateur|Une goutte de pluie brille sur le toit.
+narrateur|Victorino a encore le camion, à la table.
+narrateur|Le camion attend au bord du bois.
+narrateur|C'était l'histoire.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le camion reste à la table.</t>
+        </is>
+      </c>
+      <c r="AX40" t="inlineStr">
+        <is>
+          <t>camion</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -7961,7 +8412,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi la table, l'histoire, et le camion. Bravo, Victorino. C'est du bon travail. Le camion s'endort, une roue encore tiède. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -8101,7 +8552,14 @@
       <c r="AV41" s="2" t="inlineStr"/>
       <c r="AW41" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi la table, l'histoire, et le camion.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|Le camion s'endort, une roue encore tiède.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX41" t="inlineStr"/>
@@ -8129,7 +8587,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Sami. Il a attendu. Puis il a parlé, à la table, pendant l'histoire.</t>
+          <t>Le gobelet est jaune, un peu froid. L'eau tremble au fond, tout calme. Un reflet de fenêtre y danse. Victorino a encore le gobelet, à la table. Le gobelet fait un rond humide, sur la table. C'était l'histoire. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le gobelet reste à la table.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -8269,7 +8727,22 @@
       <c r="AV42" s="2" t="inlineStr"/>
       <c r="AW42" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Sami. Il a attendu. Puis il a parlé, à la table, pendant l'histoire.</t>
+          <t>narrateur|Le gobelet est jaune, un peu froid.
+narrateur|L'eau tremble au fond, tout calme.
+narrateur|Un reflet de fenêtre y danse.
+narrateur|Victorino a encore le gobelet, à la table.
+narrateur|Le gobelet fait un rond humide, sur la table.
+narrateur|C'était l'histoire.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le gobelet reste à la table.</t>
         </is>
       </c>
       <c r="AX42" t="inlineStr"/>
@@ -8297,7 +8770,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi la table, l'histoire, et le gobelet. Bravo, Victorino. C'est du bon travail. L'eau du gobelet ne tremble plus. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -8437,7 +8910,14 @@
       <c r="AV43" s="2" t="inlineStr"/>
       <c r="AW43" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi la table, l'histoire, et le gobelet.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|L'eau du gobelet ne tremble plus.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX43" t="inlineStr"/>
@@ -8465,7 +8945,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Barnabé attend. Puis il parle.</t>
+          <t>Papa tapote la table, tout doux. Ça fait un petit toc, comme la pluie. Moi, je chante la gouttière d'abord. Papa chante jusqu'au bout. Victorino lève la main. Il attend. Je peux chanter ? Oui. Tu as attendu. Puis on parle. Victorino chante tout bas, une petite pluie. Bravo, Victorino. On lève la main, même pour chanter. Les moufles bleues bougent un peu, au radiateur. La table rend le toc plus clair. On est encore à la table. On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -8605,7 +9085,24 @@
       <c r="AV44" s="2" t="inlineStr"/>
       <c r="AW44" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé attend. Puis il parle.</t>
+          <t>narrateur|Papa tapote la table, tout doux.
+narrateur|Ça fait un petit toc, comme la pluie.
+papa|Moi, je chante la gouttière d'abord.
+narrateur|Papa chante jusqu'au bout.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Je peux chanter ?
+maman|Oui.
+maman|Tu as attendu.
+maman|Puis on parle.
+narrateur|Victorino chante tout bas, une petite pluie.
+papa|Bravo, Victorino.
+papa|On lève la main, même pour chanter.
+narrateur|Les moufles bleues bougent un peu, au radiateur.
+narrateur|La table rend le toc plus clair.
+narrateur|On est encore à la table.
+maman|On peut attendre.
+maman|Puis on parle.</t>
         </is>
       </c>
       <c r="AX44" t="inlineStr"/>
@@ -8633,7 +9130,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre Léa, Tom, ou Sami.</t>
+          <t>Trois objets sont là, tout près. Le doudou, le camion, ou le gobelet ? On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -8801,7 +9298,10 @@
       </c>
       <c r="AW45" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre Léa, Tom, ou Sami.</t>
+          <t>narrateur|Trois objets sont là, tout près.
+papa|Le doudou, le camion, ou le gobelet ?
+maman|On peut attendre.
+maman|Puis on parle.</t>
         </is>
       </c>
       <c r="AX45" t="inlineStr"/>
@@ -8829,7 +9329,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Léa. Il a attendu. Puis il a parlé, à la table, pendant la chanson.</t>
+          <t>Le doudou est gris, un peu râpé. Une oreille est encore chaude. Il sent l'orange, tout doux. Victorino a encore le doudou, à la table. Le doudou tapote le bois, tout léger. C'était la chanson. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le doudou reste à la table.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -8969,7 +9469,22 @@
       <c r="AV46" s="2" t="inlineStr"/>
       <c r="AW46" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Léa. Il a attendu. Puis il a parlé, à la table, pendant la chanson.</t>
+          <t>narrateur|Le doudou est gris, un peu râpé.
+narrateur|Une oreille est encore chaude.
+narrateur|Il sent l'orange, tout doux.
+narrateur|Victorino a encore le doudou, à la table.
+narrateur|Le doudou tapote le bois, tout léger.
+narrateur|C'était la chanson.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le doudou reste à la table.</t>
         </is>
       </c>
       <c r="AX46" t="inlineStr"/>
@@ -8997,7 +9512,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi la table, la chanson, et le doudou. Bravo, Victorino. C'est du bon travail. Le doudou garde l'oreille chaude, tout calme. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -9137,7 +9652,14 @@
       <c r="AV47" s="2" t="inlineStr"/>
       <c r="AW47" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi la table, la chanson, et le doudou.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|Le doudou garde l'oreille chaude, tout calme.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX47" t="inlineStr"/>
@@ -9165,7 +9687,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Tom. Il a attendu. Puis il a parlé, à la table, pendant la chanson.</t>
+          <t>Le camion est rouge, tout petit. Une roue crisse, tout fin. Une goutte de pluie brille sur le toit. Victorino a encore le camion, à la table. Le camion avance d'une roue, puis s'arrête. C'était la chanson. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le camion reste à la table.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -9305,10 +9827,29 @@
       <c r="AV48" s="2" t="inlineStr"/>
       <c r="AW48" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Tom. Il a attendu. Puis il a parlé, à la table, pendant la chanson.</t>
-        </is>
-      </c>
-      <c r="AX48" t="inlineStr"/>
+          <t>narrateur|Le camion est rouge, tout petit.
+narrateur|Une roue crisse, tout fin.
+narrateur|Une goutte de pluie brille sur le toit.
+narrateur|Victorino a encore le camion, à la table.
+narrateur|Le camion avance d'une roue, puis s'arrête.
+narrateur|C'était la chanson.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le camion reste à la table.</t>
+        </is>
+      </c>
+      <c r="AX48" t="inlineStr">
+        <is>
+          <t>camion</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -9333,7 +9874,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi la table, la chanson, et le camion. Bravo, Victorino. C'est du bon travail. Le camion s'endort, une roue encore tiède. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -9473,7 +10014,14 @@
       <c r="AV49" s="2" t="inlineStr"/>
       <c r="AW49" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi la table, la chanson, et le camion.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|Le camion s'endort, une roue encore tiède.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX49" t="inlineStr"/>
@@ -9501,7 +10049,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Sami. Il a attendu. Puis il a parlé, à la table, pendant la chanson.</t>
+          <t>Le gobelet est jaune, un peu froid. L'eau tremble au fond, tout calme. Un reflet de fenêtre y danse. Victorino a encore le gobelet, à la table. Le gobelet sonne un tout petit ding. C'était la chanson. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le gobelet reste à la table.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -9641,7 +10189,22 @@
       <c r="AV50" s="2" t="inlineStr"/>
       <c r="AW50" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Sami. Il a attendu. Puis il a parlé, à la table, pendant la chanson.</t>
+          <t>narrateur|Le gobelet est jaune, un peu froid.
+narrateur|L'eau tremble au fond, tout calme.
+narrateur|Un reflet de fenêtre y danse.
+narrateur|Victorino a encore le gobelet, à la table.
+narrateur|Le gobelet sonne un tout petit ding.
+narrateur|C'était la chanson.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le gobelet reste à la table.</t>
         </is>
       </c>
       <c r="AX50" t="inlineStr"/>
@@ -9669,7 +10232,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi la table, la chanson, et le gobelet. Bravo, Victorino. C'est du bon travail. L'eau du gobelet ne tremble plus. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -9809,7 +10372,14 @@
       <c r="AV51" s="2" t="inlineStr"/>
       <c r="AW51" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi la table, la chanson, et le gobelet.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|L'eau du gobelet ne tremble plus.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX51" t="inlineStr"/>
@@ -9837,7 +10407,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Barnabé attend. Puis il parle.</t>
+          <t>Un papier blanc attend, tout lisse. Le crayon bleu a encore sa mine cassée. Moi, je dessine le bateau d'abord. Maman trace une voile, tout lentement. Victorino lève la main. Il attend. Je peux un trait ? Oui. C'est ton tour. On peut attendre. Puis on parle. Victorino pose un trait bleu, tout court. Bravo. Tu as levé la main. Le trait bleu brille, sur le bois. On est encore à la table. On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -9977,10 +10547,31 @@
       <c r="AV52" s="2" t="inlineStr"/>
       <c r="AW52" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé attend. Puis il parle.</t>
-        </is>
-      </c>
-      <c r="AX52" t="inlineStr"/>
+          <t>narrateur|Un papier blanc attend, tout lisse.
+narrateur|Le crayon bleu a encore sa mine cassée.
+maman|Moi, je dessine le bateau d'abord.
+narrateur|Maman trace une voile, tout lentement.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Je peux un trait ?
+papa|Oui.
+papa|C'est ton tour.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino pose un trait bleu, tout court.
+maman|Bravo.
+maman|Tu as levé la main.
+narrateur|Le trait bleu brille, sur le bois.
+narrateur|On est encore à la table.
+maman|On peut attendre.
+maman|Puis on parle.</t>
+        </is>
+      </c>
+      <c r="AX52" t="inlineStr">
+        <is>
+          <t>crayon</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -10005,7 +10596,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre Léa, Tom, ou Sami.</t>
+          <t>Trois objets sont là, tout près. Le doudou, le camion, ou le gobelet ? On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -10173,7 +10764,10 @@
       </c>
       <c r="AW53" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre Léa, Tom, ou Sami.</t>
+          <t>narrateur|Trois objets sont là, tout près.
+papa|Le doudou, le camion, ou le gobelet ?
+maman|On peut attendre.
+maman|Puis on parle.</t>
         </is>
       </c>
       <c r="AX53" t="inlineStr"/>
@@ -10201,7 +10795,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Léa. Il a attendu. Puis il a parlé, à la table, pendant le dessin.</t>
+          <t>Le doudou est gris, un peu râpé. Une oreille est encore chaude. Il sent l'orange, tout doux. Victorino a encore le doudou, à la table. Le doudou garde le papier, à table. C'était le dessin. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le doudou reste à la table.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -10341,7 +10935,22 @@
       <c r="AV54" s="2" t="inlineStr"/>
       <c r="AW54" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Léa. Il a attendu. Puis il a parlé, à la table, pendant le dessin.</t>
+          <t>narrateur|Le doudou est gris, un peu râpé.
+narrateur|Une oreille est encore chaude.
+narrateur|Il sent l'orange, tout doux.
+narrateur|Victorino a encore le doudou, à la table.
+narrateur|Le doudou garde le papier, à table.
+narrateur|C'était le dessin.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le doudou reste à la table.</t>
         </is>
       </c>
       <c r="AX54" t="inlineStr"/>
@@ -10369,7 +10978,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi la table, le dessin, et le doudou. Bravo, Victorino. C'est du bon travail. Le doudou garde l'oreille chaude, tout calme. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -10509,7 +11118,14 @@
       <c r="AV55" s="2" t="inlineStr"/>
       <c r="AW55" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi la table, le dessin, et le doudou.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|Le doudou garde l'oreille chaude, tout calme.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX55" t="inlineStr"/>
@@ -10537,7 +11153,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Tom. Il a attendu. Puis il a parlé, à la table, pendant le dessin.</t>
+          <t>Le camion est rouge, tout petit. Une roue crisse, tout fin. Une goutte de pluie brille sur le toit. Victorino a encore le camion, à la table. Le camion laisse une trace, à côté du trait. C'était le dessin. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le camion reste à la table.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -10677,10 +11293,29 @@
       <c r="AV56" s="2" t="inlineStr"/>
       <c r="AW56" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Tom. Il a attendu. Puis il a parlé, à la table, pendant le dessin.</t>
-        </is>
-      </c>
-      <c r="AX56" t="inlineStr"/>
+          <t>narrateur|Le camion est rouge, tout petit.
+narrateur|Une roue crisse, tout fin.
+narrateur|Une goutte de pluie brille sur le toit.
+narrateur|Victorino a encore le camion, à la table.
+narrateur|Le camion laisse une trace, à côté du trait.
+narrateur|C'était le dessin.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le camion reste à la table.</t>
+        </is>
+      </c>
+      <c r="AX56" t="inlineStr">
+        <is>
+          <t>camion</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -10705,7 +11340,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi la table, le dessin, et le camion. Bravo, Victorino. C'est du bon travail. Le camion s'endort, une roue encore tiède. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -10845,7 +11480,14 @@
       <c r="AV57" s="2" t="inlineStr"/>
       <c r="AW57" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi la table, le dessin, et le camion.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|Le camion s'endort, une roue encore tiède.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX57" t="inlineStr"/>
@@ -10873,7 +11515,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Sami. Il a attendu. Puis il a parlé, à la table, pendant le dessin.</t>
+          <t>Le gobelet est jaune, un peu froid. L'eau tremble au fond, tout calme. Un reflet de fenêtre y danse. Victorino a encore le gobelet, à la table. Le gobelet jaune éclaire le dessin. C'était le dessin. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le gobelet reste à la table.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -11013,7 +11655,22 @@
       <c r="AV58" s="2" t="inlineStr"/>
       <c r="AW58" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Sami. Il a attendu. Puis il a parlé, à la table, pendant le dessin.</t>
+          <t>narrateur|Le gobelet est jaune, un peu froid.
+narrateur|L'eau tremble au fond, tout calme.
+narrateur|Un reflet de fenêtre y danse.
+narrateur|Victorino a encore le gobelet, à la table.
+narrateur|Le gobelet jaune éclaire le dessin.
+narrateur|C'était le dessin.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le gobelet reste à la table.</t>
         </is>
       </c>
       <c r="AX58" t="inlineStr"/>
@@ -11041,7 +11698,7 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi la table, le dessin, et le gobelet. Bravo, Victorino. C'est du bon travail. L'eau du gobelet ne tremble plus. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -11181,7 +11838,14 @@
       <c r="AV59" s="2" t="inlineStr"/>
       <c r="AW59" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi la table, le dessin, et le gobelet.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|L'eau du gobelet ne tremble plus.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX59" t="inlineStr"/>
@@ -11209,7 +11873,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Près de la fenêtre, Barnabé lève la main. Il attend. Puis il parle.</t>
+          <t>Victorino s'approche de la fenêtre. La vitre est embuée, toute douce au doigt. Le bateau en papier attend sur le rebord. Dehors, la gouttière chante, tout fin. Moi, je raconte le bateau. Maman parle jusqu'au bout. Victorino lève la main. Il attend. Le bateau a une voile pliée. C'est ton tour. On a attendu. Puis on parle. Bravo. Tu as levé la main. Un trait d'eau glisse sur la vitre. Le bateau ne bouge pas.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -11349,10 +12013,29 @@
       <c r="AV60" s="2" t="inlineStr"/>
       <c r="AW60" t="inlineStr">
         <is>
-          <t>narrateur|Près de la fenêtre, Barnabé lève la main. Il attend. Puis il parle.</t>
-        </is>
-      </c>
-      <c r="AX60" t="inlineStr"/>
+          <t>narrateur|Victorino s'approche de la fenêtre.
+narrateur|La vitre est embuée, toute douce au doigt.
+narrateur|Le bateau en papier attend sur le rebord.
+narrateur|Dehors, la gouttière chante, tout fin.
+maman|Moi, je raconte le bateau.
+narrateur|Maman parle jusqu'au bout.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Le bateau a une voile pliée.
+papa|C'est ton tour.
+papa|On a attendu.
+papa|Puis on parle.
+maman|Bravo.
+maman|Tu as levé la main.
+narrateur|Un trait d'eau glisse sur la vitre.
+narrateur|Le bateau ne bouge pas.</t>
+        </is>
+      </c>
+      <c r="AX60" t="inlineStr">
+        <is>
+          <t>pluie</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -11377,7 +12060,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Près de la fenêtre, que fait Barnabé d'abord ?</t>
+          <t>Près de la fenêtre, chacun son tour. On attend, puis on parle ?</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -11533,7 +12216,8 @@
       </c>
       <c r="AW61" t="inlineStr">
         <is>
-          <t>narrateur|Près de la fenêtre, que fait Barnabé d'abord ?</t>
+          <t>narrateur|Près de la fenêtre, chacun son tour.
+maman|On attend, puis on parle ?</t>
         </is>
       </c>
       <c r="AX61" t="inlineStr"/>
@@ -11561,7 +12245,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Barnabé a levé la main. Il a attendu. Puis il a parlé.</t>
+          <t>Oui. On lève la main. On peut attendre. Puis on parle. Victorino hoche la tête. Chacun son tour. On continue, tout doux. Tu as levé la main. La gouttière chante encore, dehors.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -11705,7 +12389,15 @@
       </c>
       <c r="AW62" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé a levé la main. Il a attendu. Puis il a parlé.</t>
+          <t>maman|Oui.
+maman|On lève la main.
+maman|On peut attendre.
+maman|Puis on parle.
+narrateur|Victorino hoche la tête.
+enfant-m|Chacun son tour.
+papa|On continue, tout doux.
+papa|Tu as levé la main.
+narrateur|La gouttière chante encore, dehors.</t>
         </is>
       </c>
       <c r="AX62" t="inlineStr"/>
@@ -11733,7 +12425,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre l'histoire, la chanson, ou le dessin.</t>
+          <t>Trois choses attendent, dans la classe. L'histoire, la chanson, ou le dessin ? On lève la main. On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -11897,7 +12589,11 @@
       <c r="AV63" s="2" t="inlineStr"/>
       <c r="AW63" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre l'histoire, la chanson, ou le dessin.</t>
+          <t>narrateur|Trois choses attendent, dans la classe.
+maman|L'histoire, la chanson, ou le dessin ?
+papa|On lève la main.
+papa|On peut attendre.
+papa|Puis on parle.</t>
         </is>
       </c>
       <c r="AX63" t="inlineStr"/>
@@ -11925,7 +12621,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Barnabé attend. Puis il parle.</t>
+          <t>Maman ouvre un livre d'images. Une page sent le papier, un peu sec. Un bateau y flotte, tout blanc. Moi, je lis l'histoire d'abord. Maman lit jusqu'au bout. Victorino lève la main. Il attend. Le bateau a une voile. Oui. C'est ton tour. On peut attendre. Puis on parle. Victorino touche le papier, tout léger. Bravo. Tu as attendu. Le bateau du livre regarde le bateau du rebord. On est encore près de la fenêtre. On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -12065,10 +12761,32 @@
       <c r="AV64" s="2" t="inlineStr"/>
       <c r="AW64" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé attend. Puis il parle.</t>
-        </is>
-      </c>
-      <c r="AX64" t="inlineStr"/>
+          <t>narrateur|Maman ouvre un livre d'images.
+narrateur|Une page sent le papier, un peu sec.
+narrateur|Un bateau y flotte, tout blanc.
+maman|Moi, je lis l'histoire d'abord.
+narrateur|Maman lit jusqu'au bout.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Le bateau a une voile.
+papa|Oui.
+papa|C'est ton tour.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino touche le papier, tout léger.
+maman|Bravo.
+maman|Tu as attendu.
+narrateur|Le bateau du livre regarde le bateau du rebord.
+narrateur|On est encore près de la fenêtre.
+maman|On peut attendre.
+maman|Puis on parle.</t>
+        </is>
+      </c>
+      <c r="AX64" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -12093,7 +12811,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre Léa, Tom, ou Sami.</t>
+          <t>Trois objets sont là, tout près. Le doudou, le camion, ou le gobelet ? On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -12261,7 +12979,10 @@
       </c>
       <c r="AW65" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre Léa, Tom, ou Sami.</t>
+          <t>narrateur|Trois objets sont là, tout près.
+papa|Le doudou, le camion, ou le gobelet ?
+maman|On peut attendre.
+maman|Puis on parle.</t>
         </is>
       </c>
       <c r="AX65" t="inlineStr"/>
@@ -12289,7 +13010,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Léa. Il a attendu. Puis il a parlé, à la fenêtre, pendant l'histoire.</t>
+          <t>Le doudou est gris, un peu râpé. Une oreille est encore chaude. Il sent l'orange, tout doux. Victorino a encore le doudou, près de la fenêtre. Le doudou regarde le bateau du rebord. C'était l'histoire. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le doudou reste près de la fenêtre.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -12429,7 +13150,22 @@
       <c r="AV66" s="2" t="inlineStr"/>
       <c r="AW66" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Léa. Il a attendu. Puis il a parlé, à la fenêtre, pendant l'histoire.</t>
+          <t>narrateur|Le doudou est gris, un peu râpé.
+narrateur|Une oreille est encore chaude.
+narrateur|Il sent l'orange, tout doux.
+narrateur|Victorino a encore le doudou, près de la fenêtre.
+narrateur|Le doudou regarde le bateau du rebord.
+narrateur|C'était l'histoire.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le doudou reste près de la fenêtre.</t>
         </is>
       </c>
       <c r="AX66" t="inlineStr"/>
@@ -12457,7 +13193,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi la fenêtre, l'histoire, et le doudou. Bravo, Victorino. C'est du bon travail. Le doudou garde l'oreille chaude, tout calme. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -12597,7 +13333,14 @@
       <c r="AV67" s="2" t="inlineStr"/>
       <c r="AW67" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi la fenêtre, l'histoire, et le doudou.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|Le doudou garde l'oreille chaude, tout calme.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX67" t="inlineStr"/>
@@ -12625,7 +13368,7 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Tom. Il a attendu. Puis il a parlé, à la fenêtre, pendant l'histoire.</t>
+          <t>Le camion est rouge, tout petit. Une roue crisse, tout fin. Une goutte de pluie brille sur le toit. Victorino a encore le camion, près de la fenêtre. Le camion se gare sous le bateau en papier. C'était l'histoire. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le camion reste près de la fenêtre.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -12765,10 +13508,29 @@
       <c r="AV68" s="2" t="inlineStr"/>
       <c r="AW68" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Tom. Il a attendu. Puis il a parlé, à la fenêtre, pendant l'histoire.</t>
-        </is>
-      </c>
-      <c r="AX68" t="inlineStr"/>
+          <t>narrateur|Le camion est rouge, tout petit.
+narrateur|Une roue crisse, tout fin.
+narrateur|Une goutte de pluie brille sur le toit.
+narrateur|Victorino a encore le camion, près de la fenêtre.
+narrateur|Le camion se gare sous le bateau en papier.
+narrateur|C'était l'histoire.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le camion reste près de la fenêtre.</t>
+        </is>
+      </c>
+      <c r="AX68" t="inlineStr">
+        <is>
+          <t>camion</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -12793,7 +13555,7 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi la fenêtre, l'histoire, et le camion. Bravo, Victorino. C'est du bon travail. Le camion s'endort, une roue encore tiède. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -12933,7 +13695,14 @@
       <c r="AV69" s="2" t="inlineStr"/>
       <c r="AW69" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi la fenêtre, l'histoire, et le camion.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|Le camion s'endort, une roue encore tiède.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX69" t="inlineStr"/>
@@ -12961,7 +13730,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Sami. Il a attendu. Puis il a parlé, à la fenêtre, pendant l'histoire.</t>
+          <t>Le gobelet est jaune, un peu froid. L'eau tremble au fond, tout calme. Un reflet de fenêtre y danse. Victorino a encore le gobelet, près de la fenêtre. Le gobelet reflète la vitre embuée. C'était l'histoire. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le gobelet reste près de la fenêtre.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -13101,7 +13870,22 @@
       <c r="AV70" s="2" t="inlineStr"/>
       <c r="AW70" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Sami. Il a attendu. Puis il a parlé, à la fenêtre, pendant l'histoire.</t>
+          <t>narrateur|Le gobelet est jaune, un peu froid.
+narrateur|L'eau tremble au fond, tout calme.
+narrateur|Un reflet de fenêtre y danse.
+narrateur|Victorino a encore le gobelet, près de la fenêtre.
+narrateur|Le gobelet reflète la vitre embuée.
+narrateur|C'était l'histoire.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le gobelet reste près de la fenêtre.</t>
         </is>
       </c>
       <c r="AX70" t="inlineStr"/>
@@ -13129,7 +13913,7 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi la fenêtre, l'histoire, et le gobelet. Bravo, Victorino. C'est du bon travail. L'eau du gobelet ne tremble plus. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -13269,7 +14053,14 @@
       <c r="AV71" s="2" t="inlineStr"/>
       <c r="AW71" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi la fenêtre, l'histoire, et le gobelet.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|L'eau du gobelet ne tremble plus.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX71" t="inlineStr"/>
@@ -13297,7 +14088,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Barnabé attend. Puis il parle.</t>
+          <t>Papa tapote la table, tout doux. Ça fait un petit toc, comme la pluie. Moi, je chante la gouttière d'abord. Papa chante jusqu'au bout. Victorino lève la main. Il attend. Je peux chanter ? Oui. Tu as attendu. Puis on parle. Victorino chante tout bas, une petite pluie. Bravo, Victorino. On lève la main, même pour chanter. Les moufles bleues bougent un peu, au radiateur. La gouttière chante avec papa, dehors. On est encore près de la fenêtre. On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -13437,7 +14228,24 @@
       <c r="AV72" s="2" t="inlineStr"/>
       <c r="AW72" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé attend. Puis il parle.</t>
+          <t>narrateur|Papa tapote la table, tout doux.
+narrateur|Ça fait un petit toc, comme la pluie.
+papa|Moi, je chante la gouttière d'abord.
+narrateur|Papa chante jusqu'au bout.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Je peux chanter ?
+maman|Oui.
+maman|Tu as attendu.
+maman|Puis on parle.
+narrateur|Victorino chante tout bas, une petite pluie.
+papa|Bravo, Victorino.
+papa|On lève la main, même pour chanter.
+narrateur|Les moufles bleues bougent un peu, au radiateur.
+narrateur|La gouttière chante avec papa, dehors.
+narrateur|On est encore près de la fenêtre.
+maman|On peut attendre.
+maman|Puis on parle.</t>
         </is>
       </c>
       <c r="AX72" t="inlineStr"/>
@@ -13465,7 +14273,7 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre Léa, Tom, ou Sami.</t>
+          <t>Trois objets sont là, tout près. Le doudou, le camion, ou le gobelet ? On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -13633,7 +14441,10 @@
       </c>
       <c r="AW73" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre Léa, Tom, ou Sami.</t>
+          <t>narrateur|Trois objets sont là, tout près.
+papa|Le doudou, le camion, ou le gobelet ?
+maman|On peut attendre.
+maman|Puis on parle.</t>
         </is>
       </c>
       <c r="AX73" t="inlineStr"/>
@@ -13661,7 +14472,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Léa. Il a attendu. Puis il a parlé, à la fenêtre, pendant la chanson.</t>
+          <t>Le doudou est gris, un peu râpé. Une oreille est encore chaude. Il sent l'orange, tout doux. Victorino a encore le doudou, près de la fenêtre. Le doudou écoute la gouttière, tout près. C'était la chanson. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le doudou reste près de la fenêtre.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -13801,7 +14612,22 @@
       <c r="AV74" s="2" t="inlineStr"/>
       <c r="AW74" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Léa. Il a attendu. Puis il a parlé, à la fenêtre, pendant la chanson.</t>
+          <t>narrateur|Le doudou est gris, un peu râpé.
+narrateur|Une oreille est encore chaude.
+narrateur|Il sent l'orange, tout doux.
+narrateur|Victorino a encore le doudou, près de la fenêtre.
+narrateur|Le doudou écoute la gouttière, tout près.
+narrateur|C'était la chanson.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le doudou reste près de la fenêtre.</t>
         </is>
       </c>
       <c r="AX74" t="inlineStr"/>
@@ -13829,7 +14655,7 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi la fenêtre, la chanson, et le doudou. Bravo, Victorino. C'est du bon travail. Le doudou garde l'oreille chaude, tout calme. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -13969,7 +14795,14 @@
       <c r="AV75" s="2" t="inlineStr"/>
       <c r="AW75" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi la fenêtre, la chanson, et le doudou.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|Le doudou garde l'oreille chaude, tout calme.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX75" t="inlineStr"/>
@@ -13997,7 +14830,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Tom. Il a attendu. Puis il a parlé, à la fenêtre, pendant la chanson.</t>
+          <t>Le camion est rouge, tout petit. Une roue crisse, tout fin. Une goutte de pluie brille sur le toit. Victorino a encore le camion, près de la fenêtre. Le camion rouge brille, contre la lumière. C'était la chanson. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le camion reste près de la fenêtre.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -14137,10 +14970,29 @@
       <c r="AV76" s="2" t="inlineStr"/>
       <c r="AW76" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Tom. Il a attendu. Puis il a parlé, à la fenêtre, pendant la chanson.</t>
-        </is>
-      </c>
-      <c r="AX76" t="inlineStr"/>
+          <t>narrateur|Le camion est rouge, tout petit.
+narrateur|Une roue crisse, tout fin.
+narrateur|Une goutte de pluie brille sur le toit.
+narrateur|Victorino a encore le camion, près de la fenêtre.
+narrateur|Le camion rouge brille, contre la lumière.
+narrateur|C'était la chanson.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le camion reste près de la fenêtre.</t>
+        </is>
+      </c>
+      <c r="AX76" t="inlineStr">
+        <is>
+          <t>camion</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -14165,7 +15017,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi la fenêtre, la chanson, et le camion. Bravo, Victorino. C'est du bon travail. Le camion s'endort, une roue encore tiède. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -14305,7 +15157,14 @@
       <c r="AV77" s="2" t="inlineStr"/>
       <c r="AW77" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi la fenêtre, la chanson, et le camion.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|Le camion s'endort, une roue encore tiède.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX77" t="inlineStr"/>
@@ -14333,7 +15192,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Sami. Il a attendu. Puis il a parlé, à la fenêtre, pendant la chanson.</t>
+          <t>Le gobelet est jaune, un peu froid. L'eau tremble au fond, tout calme. Un reflet de fenêtre y danse. Victorino a encore le gobelet, près de la fenêtre. L'eau du gobelet tremble, comme la pluie. C'était la chanson. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le gobelet reste près de la fenêtre.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -14473,7 +15332,22 @@
       <c r="AV78" s="2" t="inlineStr"/>
       <c r="AW78" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Sami. Il a attendu. Puis il a parlé, à la fenêtre, pendant la chanson.</t>
+          <t>narrateur|Le gobelet est jaune, un peu froid.
+narrateur|L'eau tremble au fond, tout calme.
+narrateur|Un reflet de fenêtre y danse.
+narrateur|Victorino a encore le gobelet, près de la fenêtre.
+narrateur|L'eau du gobelet tremble, comme la pluie.
+narrateur|C'était la chanson.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le gobelet reste près de la fenêtre.</t>
         </is>
       </c>
       <c r="AX78" t="inlineStr"/>
@@ -14501,7 +15375,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi la fenêtre, la chanson, et le gobelet. Bravo, Victorino. C'est du bon travail. L'eau du gobelet ne tremble plus. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -14641,7 +15515,14 @@
       <c r="AV79" s="2" t="inlineStr"/>
       <c r="AW79" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi la fenêtre, la chanson, et le gobelet.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|L'eau du gobelet ne tremble plus.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX79" t="inlineStr"/>
@@ -14669,7 +15550,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Barnabé attend. Puis il parle.</t>
+          <t>Un papier blanc attend, tout lisse. Le crayon bleu a encore sa mine cassée. Moi, je dessine le bateau d'abord. Maman trace une voile, tout lentement. Victorino lève la main. Il attend. Je peux un trait ? Oui. C'est ton tour. On peut attendre. Puis on parle. Victorino pose un trait bleu, tout court. Bravo. Tu as levé la main. La vitre embuée garde un petit trait de doigt. On est encore près de la fenêtre. On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -14809,10 +15690,31 @@
       <c r="AV80" s="2" t="inlineStr"/>
       <c r="AW80" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé attend. Puis il parle.</t>
-        </is>
-      </c>
-      <c r="AX80" t="inlineStr"/>
+          <t>narrateur|Un papier blanc attend, tout lisse.
+narrateur|Le crayon bleu a encore sa mine cassée.
+maman|Moi, je dessine le bateau d'abord.
+narrateur|Maman trace une voile, tout lentement.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Je peux un trait ?
+papa|Oui.
+papa|C'est ton tour.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino pose un trait bleu, tout court.
+maman|Bravo.
+maman|Tu as levé la main.
+narrateur|La vitre embuée garde un petit trait de doigt.
+narrateur|On est encore près de la fenêtre.
+maman|On peut attendre.
+maman|Puis on parle.</t>
+        </is>
+      </c>
+      <c r="AX80" t="inlineStr">
+        <is>
+          <t>crayon</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -14837,7 +15739,7 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre Léa, Tom, ou Sami.</t>
+          <t>Trois objets sont là, tout près. Le doudou, le camion, ou le gobelet ? On peut attendre. Puis on parle.</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -15005,7 +15907,10 @@
       </c>
       <c r="AW81" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre Léa, Tom, ou Sami.</t>
+          <t>narrateur|Trois objets sont là, tout près.
+papa|Le doudou, le camion, ou le gobelet ?
+maman|On peut attendre.
+maman|Puis on parle.</t>
         </is>
       </c>
       <c r="AX81" t="inlineStr"/>
@@ -15033,7 +15938,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Léa. Il a attendu. Puis il a parlé, à la fenêtre, pendant le dessin.</t>
+          <t>Le doudou est gris, un peu râpé. Une oreille est encore chaude. Il sent l'orange, tout doux. Victorino a encore le doudou, près de la fenêtre. Le doudou tient le papier, près de la vitre. C'était le dessin. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le doudou reste près de la fenêtre.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -15173,7 +16078,22 @@
       <c r="AV82" s="2" t="inlineStr"/>
       <c r="AW82" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Léa. Il a attendu. Puis il a parlé, à la fenêtre, pendant le dessin.</t>
+          <t>narrateur|Le doudou est gris, un peu râpé.
+narrateur|Une oreille est encore chaude.
+narrateur|Il sent l'orange, tout doux.
+narrateur|Victorino a encore le doudou, près de la fenêtre.
+narrateur|Le doudou tient le papier, près de la vitre.
+narrateur|C'était le dessin.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le doudou reste près de la fenêtre.</t>
         </is>
       </c>
       <c r="AX82" t="inlineStr"/>
@@ -15201,7 +16121,7 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi la fenêtre, le dessin, et le doudou. Bravo, Victorino. C'est du bon travail. Le doudou garde l'oreille chaude, tout calme. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -15341,7 +16261,14 @@
       <c r="AV83" s="2" t="inlineStr"/>
       <c r="AW83" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi la fenêtre, le dessin, et le doudou.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|Le doudou garde l'oreille chaude, tout calme.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX83" t="inlineStr"/>
@@ -15369,7 +16296,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Tom. Il a attendu. Puis il a parlé, à la fenêtre, pendant le dessin.</t>
+          <t>Le camion est rouge, tout petit. Une roue crisse, tout fin. Une goutte de pluie brille sur le toit. Victorino a encore le camion, près de la fenêtre. Le camion suit le trait, vers le rebord. C'était le dessin. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le camion reste près de la fenêtre.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -15509,10 +16436,29 @@
       <c r="AV84" s="2" t="inlineStr"/>
       <c r="AW84" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Tom. Il a attendu. Puis il a parlé, à la fenêtre, pendant le dessin.</t>
-        </is>
-      </c>
-      <c r="AX84" t="inlineStr"/>
+          <t>narrateur|Le camion est rouge, tout petit.
+narrateur|Une roue crisse, tout fin.
+narrateur|Une goutte de pluie brille sur le toit.
+narrateur|Victorino a encore le camion, près de la fenêtre.
+narrateur|Le camion suit le trait, vers le rebord.
+narrateur|C'était le dessin.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le camion reste près de la fenêtre.</t>
+        </is>
+      </c>
+      <c r="AX84" t="inlineStr">
+        <is>
+          <t>camion</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -15537,7 +16483,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi la fenêtre, le dessin, et le camion. Bravo, Victorino. C'est du bon travail. Le camion s'endort, une roue encore tiède. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -15677,7 +16623,14 @@
       <c r="AV85" s="2" t="inlineStr"/>
       <c r="AW85" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi la fenêtre, le dessin, et le camion.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|Le camion s'endort, une roue encore tiède.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX85" t="inlineStr"/>
@@ -15705,7 +16658,7 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Barnabé rejoint Sami. Il a attendu. Puis il a parlé, à la fenêtre, pendant le dessin.</t>
+          <t>Le gobelet est jaune, un peu froid. L'eau tremble au fond, tout calme. Un reflet de fenêtre y danse. Victorino a encore le gobelet, près de la fenêtre. Le gobelet pose une ombre ronde, sur le dessin. C'était le dessin. On peut attendre. Puis on parle. Victorino lève la main. Il attend. Merci, papa. Bravo. Tu as attendu. Puis tu as parlé. C'est du bon travail, Victorino. Le gobelet reste près de la fenêtre.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -15845,7 +16798,22 @@
       <c r="AV86" s="2" t="inlineStr"/>
       <c r="AW86" t="inlineStr">
         <is>
-          <t>narrateur|Barnabé rejoint Sami. Il a attendu. Puis il a parlé, à la fenêtre, pendant le dessin.</t>
+          <t>narrateur|Le gobelet est jaune, un peu froid.
+narrateur|L'eau tremble au fond, tout calme.
+narrateur|Un reflet de fenêtre y danse.
+narrateur|Victorino a encore le gobelet, près de la fenêtre.
+narrateur|Le gobelet pose une ombre ronde, sur le dessin.
+narrateur|C'était le dessin.
+papa|On peut attendre.
+papa|Puis on parle.
+narrateur|Victorino lève la main.
+narrateur|Il attend.
+enfant-m|Merci, papa.
+maman|Bravo.
+maman|Tu as attendu.
+maman|Puis tu as parlé.
+papa|C'est du bon travail, Victorino.
+narrateur|Le gobelet reste près de la fenêtre.</t>
         </is>
       </c>
       <c r="AX86" t="inlineStr"/>
@@ -15873,7 +16841,7 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Tu as attendu. Puis tu as parlé. Victorino a choisi la fenêtre, le dessin, et le gobelet. Bravo, Victorino. C'est du bon travail. L'eau du gobelet ne tremble plus. Les moufles bleues sont sèches, maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -16013,7 +16981,14 @@
       <c r="AV87" s="2" t="inlineStr"/>
       <c r="AW87" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>maman|Tu as attendu.
+maman|Puis tu as parlé.
+narrateur|Victorino a choisi la fenêtre, le dessin, et le gobelet.
+papa|Bravo, Victorino.
+papa|C'est du bon travail.
+narrateur|L'eau du gobelet ne tremble plus.
+narrateur|Les moufles bleues sont sèches, maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX87" t="inlineStr"/>
@@ -16035,7 +17010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16129,6 +17104,13 @@
       <c r="A13" t="inlineStr">
         <is>
           <t>F-AUD-007 colonne sons ; vide = silence ; jamais parler dans le bruit</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-NAR-019): TREE-COL-031 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-031.xlsx
+++ b/stories/arbres/TREE-COL-031.xlsx
@@ -2926,17 +2926,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Le soir, le radiateur tic plus lent, dans le salon. Raconte-nous le voyage, jusqu'au bout. Le doudou a fait le quai, et le bateau a copié la page. Bravo. Nous t'avons entendu sans te couper. Les moufles bleues sont chaudes, sèches, un peu rêche. Le bateau sèche contre la patte du doudou, sur la serviette. Une oreille garde une petite tache d'eau, presque invisible.</t>
+          <t>Le soir, le radiateur tic plus lent, dans le salon. Raconte-nous le voyage, jusqu'au bout. Le doudou a fait le quai, et le bateau a copié la page. Nous t'avons entendu sans te couper. Les moufles bleues sont chaudes, sèches, un peu rêche. Le bateau sèche contre la patte du doudou, sur la serviette. Une oreille garde une petite tache d'eau, presque invisible.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le soir, le radiateur tic plus lent, dans le salon. Raconte-nous le voyage, jusqu'au bout. Le doudou a fait le quai, et le bateau a copié la page. Bravo. Nous t'avons entendu sans te couper. Les &lt;emphasis level="moderate"&gt;moufles&lt;/emphasis&gt; bleues sont chaudes, sèches, un peu rêche. Le bateau sèche contre la patte du doudou, sur la serviette. Une oreille garde une petite tache d'eau, presque invisible.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le soir, le radiateur tic plus lent, dans le salon. Raconte-nous le voyage, jusqu'au bout. Le doudou a fait le quai, et le bateau a copié la page. Nous t'avons entendu sans te couper. Les &lt;emphasis level="moderate"&gt;moufles&lt;/emphasis&gt; bleues sont chaudes, sèches, un peu rêche. Le bateau sèche contre la patte du doudou, sur la serviette. Une oreille garde une petite tache d'eau, presque invisible.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le soir, le radiateur tic plus lent, dans le salon. Raconte-nous le voyage, jusqu'au bout. Le doudou a fait le quai, et le bateau a copié la page. Bravo. Nous t'avons entendu sans te couper. Les &lt;emphasis&gt;moufles&lt;/emphasis&gt; bleues sont chaudes, sèches, un peu rêche. Le bateau sèche contre la patte du doudou, sur la serviette. Une oreille garde une petite tache d'eau, presque invisible.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le soir, le radiateur tic plus lent, dans le salon. Raconte-nous le voyage, jusqu'au bout. Le doudou a fait le quai, et le bateau a copié la page. Nous t'avons entendu sans te couper. Les &lt;emphasis&gt;moufles&lt;/emphasis&gt; bleues sont chaudes, sèches, un peu rêche. Le bateau sèche contre la patte du doudou, sur la serviette. Une oreille garde une petite tache d'eau, presque invisible.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -3077,7 +3077,6 @@
           <t>narrateur|Le soir, le radiateur tic plus lent, dans le salon.
 maman|Raconte-nous le voyage, jusqu'au bout.
 enfant-m|Le doudou a fait le quai, et le bateau a copié la page.
-papa|Bravo.
 papa|Nous t'avons entendu sans te couper.
 narrateur|Les moufles bleues sont chaudes, sèches, un peu rêche.
 narrateur|Le bateau sèche contre la patte du doudou, sur la serviette.
@@ -4442,17 +4441,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Le radiateur tic comme un cinquième toc, plus doux. Chante-nous les quatre coups, jusqu'au dernier. Le doudou a attendu le quatrième, et le bateau aussi. Bravo. Ton capitaine a des oreilles patientes. Les moufles bougent à peine, sèches, au-dessus du métal. Le bateau sèche contre l'oreille, une voile un peu rêche. Une tache d'eau s'efface sur le gris du doudou.</t>
+          <t>Le radiateur tic comme un cinquième toc, plus doux. Chante-nous les quatre coups, jusqu'au dernier. Le doudou a attendu le quatrième, et le bateau aussi. Ton capitaine a des oreilles patientes. Les moufles bougent à peine, sèches, au-dessus du métal. Le bateau sèche contre l'oreille, une voile un peu rêche. Une tache d'eau s'efface sur le gris du doudou.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le radiateur tic comme un cinquième toc, plus doux. Chante-nous les quatre coups, jusqu'au dernier. Le doudou a attendu le quatrième, et le bateau aussi. Bravo. Ton capitaine a des oreilles patientes. Les &lt;emphasis level="moderate"&gt;moufles&lt;/emphasis&gt; bougent à peine, sèches, au-dessus du métal. Le bateau sèche contre l'oreille, une voile un peu rêche. Une tache d'eau s'efface sur le gris du doudou.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le radiateur tic comme un cinquième toc, plus doux. Chante-nous les quatre coups, jusqu'au dernier. Le doudou a attendu le quatrième, et le bateau aussi. Ton capitaine a des oreilles patientes. Les &lt;emphasis level="moderate"&gt;moufles&lt;/emphasis&gt; bougent à peine, sèches, au-dessus du métal. Le bateau sèche contre l'oreille, une voile un peu rêche. Une tache d'eau s'efface sur le gris du doudou.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le radiateur tic comme un cinquième toc, plus doux. Chante-nous les quatre coups, jusqu'au dernier. Le doudou a attendu le quatrième, et le bateau aussi. Bravo. Ton capitaine a des oreilles patientes. Les &lt;emphasis&gt;moufles&lt;/emphasis&gt; bougent à peine, sèches, au-dessus du métal. Le bateau sèche contre l'oreille, une voile un peu rêche. Une tache d'eau s'efface sur le gris du doudou.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le radiateur tic comme un cinquième toc, plus doux. Chante-nous les quatre coups, jusqu'au dernier. Le doudou a attendu le quatrième, et le bateau aussi. Ton capitaine a des oreilles patientes. Les &lt;emphasis&gt;moufles&lt;/emphasis&gt; bougent à peine, sèches, au-dessus du métal. Le bateau sèche contre l'oreille, une voile un peu rêche. Une tache d'eau s'efface sur le gris du doudou.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -4593,7 +4592,6 @@
           <t>narrateur|Le radiateur tic comme un cinquième toc, plus doux.
 papa|Chante-nous les quatre coups, jusqu'au dernier.
 enfant-m|Le doudou a attendu le quatrième, et le bateau aussi.
-maman|Bravo.
 maman|Ton capitaine a des oreilles patientes.
 narrateur|Les moufles bougent à peine, sèches, au-dessus du métal.
 narrateur|Le bateau sèche contre l'oreille, une voile un peu rêche.
@@ -5954,17 +5952,17 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>La lumière du salon baisse. Le radiateur garde sa rondeur. Dis-nous le phare, sans rien presser. Le doudou tenait le crayon, et le bateau s'est arrêté au bleu. Bravo. Le trait a eu le temps de sécher. Les moufles, sèches, ont un fil de laine relevé. Le bateau sèche sous la patte, ligne bleue vers le zinc. Le crayon repose, mine vers le haut, loin de l'eau.</t>
+          <t>La lumière du salon baisse. Le radiateur garde sa rondeur. Dis-nous le phare, sans rien presser. Le doudou tenait le crayon, et le bateau s'est arrêté au bleu. Le trait a eu le temps de sécher. Les moufles, sèches, ont un fil de laine relevé. Le bateau sèche sous la patte, ligne bleue vers le zinc. Le crayon repose, mine vers le haut, loin de l'eau.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La lumière du salon baisse. Le radiateur garde sa rondeur. Dis-nous le phare, sans rien presser. Le doudou tenait le crayon, et le bateau s'est arrêté au bleu. Bravo. Le trait a eu le temps de sécher. Les &lt;emphasis level="moderate"&gt;moufles&lt;/emphasis&gt;, sèches, ont un fil de laine relevé. Le bateau sèche sous la patte, ligne bleue vers le zinc. Le crayon repose, mine vers le haut, loin de l'eau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La lumière du salon baisse. Le radiateur garde sa rondeur. Dis-nous le phare, sans rien presser. Le doudou tenait le crayon, et le bateau s'est arrêté au bleu. Le trait a eu le temps de sécher. Les &lt;emphasis level="moderate"&gt;moufles&lt;/emphasis&gt;, sèches, ont un fil de laine relevé. Le bateau sèche sous la patte, ligne bleue vers le zinc. Le crayon repose, mine vers le haut, loin de l'eau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La lumière du salon baisse. Le radiateur garde sa rondeur. Dis-nous le phare, sans rien presser. Le doudou tenait le crayon, et le bateau s'est arrêté au bleu. Bravo. Le trait a eu le temps de sécher. Les &lt;emphasis&gt;moufles&lt;/emphasis&gt;, sèches, ont un fil de laine relevé. Le bateau sèche sous la patte, ligne bleue vers le zinc. Le crayon repose, mine vers le haut, loin de l'eau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La lumière du salon baisse. Le radiateur garde sa rondeur. Dis-nous le phare, sans rien presser. Le doudou tenait le crayon, et le bateau s'est arrêté au bleu. Le trait a eu le temps de sécher. Les &lt;emphasis&gt;moufles&lt;/emphasis&gt;, sèches, ont un fil de laine relevé. Le bateau sèche sous la patte, ligne bleue vers le zinc. Le crayon repose, mine vers le haut, loin de l'eau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -6106,7 +6104,6 @@
 narrateur|Le radiateur garde sa rondeur.
 maman|Dis-nous le phare, sans rien presser.
 enfant-m|Le doudou tenait le crayon, et le bateau s'est arrêté au bleu.
-papa|Bravo.
 papa|Le trait a eu le temps de sécher.
 narrateur|Les moufles, sèches, ont un fil de laine relevé.
 narrateur|Le bateau sèche sous la patte, ligne bleue vers le zinc.
@@ -7266,17 +7263,17 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Oui. Il a attendu l'assiette. Maman pose la pelure sur le bord, hors du plat. Maintenant, le voyage a de la place. La voile s'est plissée. Il faut l'aider. Merci d'avoir laissé finir l'orange. Le bois de la table brille, un peu collant. Le bateau attend au bord, plus droit.</t>
+          <t>Oui. Il a attendu l'assiette. Maman pose la pelure sur le bord, hors du plat. Maintenant, le voyage a de la place. La voile s'est plissée. On peut l'aider. Merci d'avoir laissé finir l'orange. Le bois de la table brille, un peu collant. Le bateau attend au bord, plus droit.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Oui. Il a attendu l'assiette. Maman pose la pelure sur le bord, hors du plat. Maintenant, le voyage a de la place. La voile s'est plissée. Il faut l'aider. Merci d'avoir laissé finir l'&lt;emphasis level="moderate"&gt;orange&lt;/emphasis&gt;. Le bois de la table brille, un peu collant. Le bateau attend au bord, plus droit.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Oui. Il a attendu l'assiette. Maman pose la pelure sur le bord, hors du plat. Maintenant, le voyage a de la place. La voile s'est plissée. On peut l'aider. Merci d'avoir laissé finir l'&lt;emphasis level="moderate"&gt;orange&lt;/emphasis&gt;. Le bois de la table brille, un peu collant. Le bateau attend au bord, plus droit.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Oui. Il a attendu l'assiette. Maman pose la pelure sur le bord, hors du plat. Maintenant, le voyage a de la place. La voile s'est plissée. Il faut l'aider. Merci d'avoir laissé finir l'&lt;emphasis&gt;orange&lt;/emphasis&gt;. Le bois de la table brille, un peu collant. Le bateau attend au bord, plus droit. [pause]</t>
+          <t>Oui. Il a attendu l'assiette. Maman pose la pelure sur le bord, hors du plat. Maintenant, le voyage a de la place. La voile s'est plissée. On peut l'aider. Merci d'avoir laissé finir l'&lt;emphasis&gt;orange&lt;/emphasis&gt;. Le bois de la table brille, un peu collant. Le bateau attend au bord, plus droit. [pause]</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -7415,7 +7412,7 @@
 narrateur|Maman pose la pelure sur le bord, hors du plat.
 maman|Maintenant, le voyage a de la place.
 enfant-m|La voile s'est plissée.
-enfant-m|Il faut l'aider.
+enfant-m|On peut l'aider.
 papa|Merci d'avoir laissé finir l'orange.
 narrateur|Le bois de la table brille, un peu collant.
 narrateur|Le bateau attend au bord, plus droit.</t>
@@ -8221,17 +8218,17 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Le soir, l'orange a disparu. Il reste son parfum sur le bois. On t'écoute : l'île, puis le spectateur. Le doudou a regardé, et le bateau a tourné autour de l'orange. Bravo. La page a eu sa fin, et le tour aussi. Les moufles, près du radiateur, sont deux coques chaudes. Le bateau sèche contre la patte, sur la chaise. Une miette d'orange orpheline brille sur la table.</t>
+          <t>Le soir, l'orange a disparu. Il reste son parfum sur le bois. On t'écoute : l'île, puis le spectateur. Le doudou a regardé, et le bateau a tourné autour de l'orange. La page a eu sa fin, et le tour aussi. Les moufles, près du radiateur, sont deux coques chaudes. Le bateau sèche contre la patte, sur la chaise. Une miette d'orange orpheline brille sur la table.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le soir, l'orange a disparu. Il reste son parfum sur le bois. On t'écoute : l'île, puis le spectateur. Le doudou a regardé, et le bateau a tourné autour de l'orange. Bravo. La page a eu sa fin, et le tour aussi. Les &lt;emphasis level="moderate"&gt;moufles&lt;/emphasis&gt;, près du radiateur, sont deux coques chaudes. Le bateau sèche contre la patte, sur la chaise. Une miette d'orange orpheline brille sur la table.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le soir, l'orange a disparu. Il reste son parfum sur le bois. On t'écoute : l'île, puis le spectateur. Le doudou a regardé, et le bateau a tourné autour de l'orange. La page a eu sa fin, et le tour aussi. Les &lt;emphasis level="moderate"&gt;moufles&lt;/emphasis&gt;, près du radiateur, sont deux coques chaudes. Le bateau sèche contre la patte, sur la chaise. Une miette d'orange orpheline brille sur la table.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le soir, l'orange a disparu. Il reste son parfum sur le bois. On t'écoute : l'île, puis le spectateur. Le doudou a regardé, et le bateau a tourné autour de l'orange. Bravo. La page a eu sa fin, et le tour aussi. Les &lt;emphasis&gt;moufles&lt;/emphasis&gt;, près du radiateur, sont deux coques chaudes. Le bateau sèche contre la patte, sur la chaise. Une miette d'orange orpheline brille sur la table.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le soir, l'orange a disparu. Il reste son parfum sur le bois. On t'écoute : l'île, puis le spectateur. Le doudou a regardé, et le bateau a tourné autour de l'orange. La page a eu sa fin, et le tour aussi. Les &lt;emphasis&gt;moufles&lt;/emphasis&gt;, près du radiateur, sont deux coques chaudes. Le bateau sèche contre la patte, sur la chaise. Une miette d'orange orpheline brille sur la table.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -8373,7 +8370,6 @@
 narrateur|Il reste son parfum sur le bois.
 maman|On t'écoute : l'île, puis le spectateur.
 enfant-m|Le doudou a regardé, et le bateau a tourné autour de l'orange.
-papa|Bravo.
 papa|La page a eu sa fin, et le tour aussi.
 narrateur|Les moufles, près du radiateur, sont deux coques chaudes.
 narrateur|Le bateau sèche contre la patte, sur la chaise.
@@ -9735,17 +9731,17 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Les cuillères sont silencieuses, dans leur tiroir. On t'écoute : les trois coups, puis le museau. Le doudou a dirigé au troisième, et le bateau s'est amarré. Bravo. L'orchestre a eu sa mesure entière. Les moufles sèches tapent un tout petit tic, contre le métal. Le bateau sèche sous le museau, sur la nappe. Une oreille garde le souvenir des trois coups, un pli.</t>
+          <t>Les cuillères sont silencieuses, dans leur tiroir. On t'écoute : les trois coups, puis le museau. Le doudou a dirigé au troisième, et le bateau s'est amarré. L'orchestre a eu sa mesure entière. Les moufles sèches tapent un tout petit tic, contre le métal. Le bateau sèche sous le museau, sur la nappe. Une oreille garde le souvenir des trois coups, un pli.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les cuillères sont silencieuses, dans leur tiroir. On t'écoute : les trois coups, puis le museau. Le doudou a dirigé au troisième, et le bateau s'est amarré. Bravo. L'orchestre a eu sa mesure entière. Les &lt;emphasis level="moderate"&gt;moufles&lt;/emphasis&gt; sèches tapent un tout petit tic, contre le métal. Le bateau sèche sous le museau, sur la nappe. Une oreille garde le souvenir des trois coups, un pli.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les cuillères sont silencieuses, dans leur tiroir. On t'écoute : les trois coups, puis le museau. Le doudou a dirigé au troisième, et le bateau s'est amarré. L'orchestre a eu sa mesure entière. Les &lt;emphasis level="moderate"&gt;moufles&lt;/emphasis&gt; sèches tapent un tout petit tic, contre le métal. Le bateau sèche sous le museau, sur la nappe. Une oreille garde le souvenir des trois coups, un pli.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les cuillères sont silencieuses, dans leur tiroir. On t'écoute : les trois coups, puis le museau. Le doudou a dirigé au troisième, et le bateau s'est amarré. Bravo. L'orchestre a eu sa mesure entière. Les &lt;emphasis&gt;moufles&lt;/emphasis&gt; sèches tapent un tout petit tic, contre le métal. Le bateau sèche sous le museau, sur la nappe. Une oreille garde le souvenir des trois coups, un pli.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les cuillères sont silencieuses, dans leur tiroir. On t'écoute : les trois coups, puis le museau. Le doudou a dirigé au troisième, et le bateau s'est amarré. L'orchestre a eu sa mesure entière. Les &lt;emphasis&gt;moufles&lt;/emphasis&gt; sèches tapent un tout petit tic, contre le métal. Le bateau sèche sous le museau, sur la nappe. Une oreille garde le souvenir des trois coups, un pli.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -9886,7 +9882,6 @@
           <t>narrateur|Les cuillères sont silencieuses, dans leur tiroir.
 papa|On t'écoute : les trois coups, puis le museau.
 enfant-m|Le doudou a dirigé au troisième, et le bateau s'est amarré.
-maman|Bravo.
 maman|L'orchestre a eu sa mesure entière.
 narrateur|Les moufles sèches tapent un tout petit tic, contre le métal.
 narrateur|Le bateau sèche sous le museau, sur la nappe.
@@ -11247,17 +11242,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>La lampe de la table fait un rond jaune sur le bois. Raconte le nez bleu, puis le quai. Le doudou a un grade, et le bateau s'est arrêté à la ligne. Bravo. Tu as laissé finir le trait. Les moufles, au radiateur, sont deux drapeaux bleus au repos. Le bateau sèche sous le nez, un point pâle pour phare. Le torchon sèche aussi, petit ciel oublié.</t>
+          <t>La lampe de la table fait un rond jaune sur le bois. Raconte le nez bleu, puis le quai. Le doudou a un grade, et le bateau s'est arrêté à la ligne. Tu as laissé finir le trait. Les moufles, au radiateur, sont deux drapeaux bleus au repos. Le bateau sèche sous le nez, un point pâle pour phare. Le torchon sèche aussi, petit ciel oublié.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La lampe de la table fait un rond jaune sur le bois. Raconte le nez bleu, puis le quai. Le doudou a un grade, et le bateau s'est arrêté à la ligne. Bravo. Tu as laissé finir le trait. Les &lt;emphasis level="moderate"&gt;moufles&lt;/emphasis&gt;, au radiateur, sont deux drapeaux bleus au repos. Le bateau sèche sous le nez, un point pâle pour phare. Le torchon sèche aussi, petit ciel oublié.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La lampe de la table fait un rond jaune sur le bois. Raconte le nez bleu, puis le quai. Le doudou a un grade, et le bateau s'est arrêté à la ligne. Tu as laissé finir le trait. Les &lt;emphasis level="moderate"&gt;moufles&lt;/emphasis&gt;, au radiateur, sont deux drapeaux bleus au repos. Le bateau sèche sous le nez, un point pâle pour phare. Le torchon sèche aussi, petit ciel oublié.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La lampe de la table fait un rond jaune sur le bois. Raconte le nez bleu, puis le quai. Le doudou a un grade, et le bateau s'est arrêté à la ligne. Bravo. Tu as laissé finir le trait. Les &lt;emphasis&gt;moufles&lt;/emphasis&gt;, au radiateur, sont deux drapeaux bleus au repos. Le bateau sèche sous le nez, un point pâle pour phare. Le torchon sèche aussi, petit ciel oublié.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La lampe de la table fait un rond jaune sur le bois. Raconte le nez bleu, puis le quai. Le doudou a un grade, et le bateau s'est arrêté à la ligne. Tu as laissé finir le trait. Les &lt;emphasis&gt;moufles&lt;/emphasis&gt;, au radiateur, sont deux drapeaux bleus au repos. Le bateau sèche sous le nez, un point pâle pour phare. Le torchon sèche aussi, petit ciel oublié.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -11398,7 +11393,6 @@
           <t>narrateur|La lampe de la table fait un rond jaune sur le bois.
 maman|Raconte le nez bleu, puis le quai.
 enfant-m|Le doudou a un grade, et le bateau s'est arrêté à la ligne.
-papa|Bravo.
 papa|Tu as laissé finir le trait.
 narrateur|Les moufles, au radiateur, sont deux drapeaux bleus au repos.
 narrateur|Le bateau sèche sous le nez, un point pâle pour phare.
@@ -13515,17 +13509,17 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>La gouttière se tait. Il reste des perles aux bords du toit. Raconte les deux voiles, depuis le glissement. Le doudou a comparé, et le vrai bateau a levé sa voile. Bravo. Le témoin a attendu la page. Les moufles, au salon, sont sèches, un peu plus petites. Le bateau sèche contre la patte, face à la vitre noire. Le livre est fermé, les deux voiles rangées dans la tête.</t>
+          <t>La gouttière se tait. Il reste des perles aux bords du toit. Raconte les deux voiles, depuis le glissement. Le doudou a comparé, et le vrai bateau a levé sa voile. Le témoin a attendu la page. Les moufles, au salon, sont sèches, un peu plus petites. Le bateau sèche contre la patte, face à la vitre noire. Le livre est fermé, les deux voiles rangées dans la tête.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La gouttière se tait. Il reste des perles aux bords du toit. Raconte les deux voiles, depuis le glissement. Le doudou a comparé, et le vrai bateau a levé sa voile. Bravo. Le témoin a attendu la page. Les &lt;emphasis level="moderate"&gt;moufles&lt;/emphasis&gt;, au salon, sont sèches, un peu plus petites. Le bateau sèche contre la patte, face à la vitre noire. Le livre est fermé, les deux voiles rangées dans la tête.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La gouttière se tait. Il reste des perles aux bords du toit. Raconte les deux voiles, depuis le glissement. Le doudou a comparé, et le vrai bateau a levé sa voile. Le témoin a attendu la page. Les &lt;emphasis level="moderate"&gt;moufles&lt;/emphasis&gt;, au salon, sont sèches, un peu plus petites. Le bateau sèche contre la patte, face à la vitre noire. Le livre est fermé, les deux voiles rangées dans la tête.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La gouttière se tait. Il reste des perles aux bords du toit. Raconte les deux voiles, depuis le glissement. Le doudou a comparé, et le vrai bateau a levé sa voile. Bravo. Le témoin a attendu la page. Les &lt;emphasis&gt;moufles&lt;/emphasis&gt;, au salon, sont sèches, un peu plus petites. Le bateau sèche contre la patte, face à la vitre noire. Le livre est fermé, les deux voiles rangées dans la tête.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La gouttière se tait. Il reste des perles aux bords du toit. Raconte les deux voiles, depuis le glissement. Le doudou a comparé, et le vrai bateau a levé sa voile. Le témoin a attendu la page. Les &lt;emphasis&gt;moufles&lt;/emphasis&gt;, au salon, sont sèches, un peu plus petites. Le bateau sèche contre la patte, face à la vitre noire. Le livre est fermé, les deux voiles rangées dans la tête.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -13667,7 +13661,6 @@
 narrateur|Il reste des perles aux bords du toit.
 maman|Raconte les deux voiles, depuis le glissement.
 enfant-m|Le doudou a comparé, et le vrai bateau a levé sa voile.
-papa|Bravo.
 papa|Le témoin a attendu la page.
 narrateur|Les moufles, au salon, sont sèches, un peu plus petites.
 narrateur|Le bateau sèche contre la patte, face à la vitre noire.
@@ -15028,17 +15021,17 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Le tuyau s'endort. Il reste un goutte-à-goutte, très loin. Chante-nous la courte, puis la longue. Le doudou a entendu la longue, et le bateau est parti avec. Bravo. Ton chœur n'a pas sauté la mesure. Les moufles, sèches, ont un pompon un peu raide. Le bateau sèche contre l'oreille, pleine de tuyau. La vitre garde un halo, là où l'oreille s'était collée.</t>
+          <t>Le tuyau s'endort. Il reste un goutte-à-goutte, très loin. Chante-nous la courte, puis la longue. Le doudou a entendu la longue, et le bateau est parti avec. Ton chœur n'a pas sauté la mesure. Les moufles, sèches, ont un pompon un peu raide. Le bateau sèche contre l'oreille, pleine de tuyau. La vitre garde un halo, là où l'oreille s'était collée.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le tuyau s'endort. Il reste un goutte-à-goutte, très loin. Chante-nous la courte, puis la longue. Le doudou a entendu la longue, et le bateau est parti avec. Bravo. Ton chœur n'a pas sauté la mesure. Les &lt;emphasis level="moderate"&gt;moufles&lt;/emphasis&gt;, sèches, ont un pompon un peu raide. Le bateau sèche contre l'oreille, pleine de tuyau. La vitre garde un halo, là où l'oreille s'était collée.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le tuyau s'endort. Il reste un goutte-à-goutte, très loin. Chante-nous la courte, puis la longue. Le doudou a entendu la longue, et le bateau est parti avec. Ton chœur n'a pas sauté la mesure. Les &lt;emphasis level="moderate"&gt;moufles&lt;/emphasis&gt;, sèches, ont un pompon un peu raide. Le bateau sèche contre l'oreille, pleine de tuyau. La vitre garde un halo, là où l'oreille s'était collée.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le tuyau s'endort. Il reste un goutte-à-goutte, très loin. Chante-nous la courte, puis la longue. Le doudou a entendu la longue, et le bateau est parti avec. Bravo. Ton chœur n'a pas sauté la mesure. Les &lt;emphasis&gt;moufles&lt;/emphasis&gt;, sèches, ont un pompon un peu raide. Le bateau sèche contre l'oreille, pleine de tuyau. La vitre garde un halo, là où l'oreille s'était collée.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le tuyau s'endort. Il reste un goutte-à-goutte, très loin. Chante-nous la courte, puis la longue. Le doudou a entendu la longue, et le bateau est parti avec. Ton chœur n'a pas sauté la mesure. Les &lt;emphasis&gt;moufles&lt;/emphasis&gt;, sèches, ont un pompon un peu raide. Le bateau sèche contre l'oreille, pleine de tuyau. La vitre garde un halo, là où l'oreille s'était collée.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -15180,7 +15173,6 @@
 narrateur|Il reste un goutte-à-goutte, très loin.
 papa|Chante-nous la courte, puis la longue.
 enfant-m|Le doudou a entendu la longue, et le bateau est parti avec.
-maman|Bravo.
 maman|Ton chœur n'a pas sauté la mesure.
 narrateur|Les moufles, sèches, ont un pompon un peu raide.
 narrateur|Le bateau sèche contre l'oreille, pleine de tuyau.
@@ -16537,17 +16529,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>La buée est partie. Le trait de doigt est devenu un fantôme. Raconte la fenêtre du capitaine, puis le quai. Le doudou a sa fenêtre, et le bateau a attendu le bleu. Bravo. Le quai a eu le temps de se fermer. Les moufles, sèches, sont rentrées dans le tiroir du banc. Le bateau sèche contre la patte, face au verre noir. Le fantôme du doigt reste, à peine, au ras du rebord.</t>
+          <t>La buée est partie. Le trait de doigt est devenu un fantôme. Raconte la fenêtre du capitaine, puis le quai. Le doudou a sa fenêtre, et le bateau a attendu le bleu. Le quai a eu le temps de se fermer. Les moufles, sèches, sont rentrées dans le tiroir du banc. Le bateau sèche contre la patte, face au verre noir. Le fantôme du doigt reste, à peine, au ras du rebord.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La buée est partie. Le trait de doigt est devenu un fantôme. Raconte la fenêtre du capitaine, puis le quai. Le doudou a sa fenêtre, et le bateau a attendu le bleu. Bravo. Le quai a eu le temps de se fermer. Les &lt;emphasis level="moderate"&gt;moufles&lt;/emphasis&gt;, sèches, sont rentrées dans le tiroir du banc. Le bateau sèche contre la patte, face au verre noir. Le fantôme du doigt reste, à peine, au ras du rebord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La buée est partie. Le trait de doigt est devenu un fantôme. Raconte la fenêtre du capitaine, puis le quai. Le doudou a sa fenêtre, et le bateau a attendu le bleu. Le quai a eu le temps de se fermer. Les &lt;emphasis level="moderate"&gt;moufles&lt;/emphasis&gt;, sèches, sont rentrées dans le tiroir du banc. Le bateau sèche contre la patte, face au verre noir. Le fantôme du doigt reste, à peine, au ras du rebord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La buée est partie. Le trait de doigt est devenu un fantôme. Raconte la fenêtre du capitaine, puis le quai. Le doudou a sa fenêtre, et le bateau a attendu le bleu. Bravo. Le quai a eu le temps de se fermer. Les &lt;emphasis&gt;moufles&lt;/emphasis&gt;, sèches, sont rentrées dans le tiroir du banc. Le bateau sèche contre la patte, face au verre noir. Le fantôme du doigt reste, à peine, au ras du rebord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La buée est partie. Le trait de doigt est devenu un fantôme. Raconte la fenêtre du capitaine, puis le quai. Le doudou a sa fenêtre, et le bateau a attendu le bleu. Le quai a eu le temps de se fermer. Les &lt;emphasis&gt;moufles&lt;/emphasis&gt;, sèches, sont rentrées dans le tiroir du banc. Le bateau sèche contre la patte, face au verre noir. Le fantôme du doigt reste, à peine, au ras du rebord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -16689,7 +16681,6 @@
 narrateur|Le trait de doigt est devenu un fantôme.
 maman|Raconte la fenêtre du capitaine, puis le quai.
 enfant-m|Le doudou a sa fenêtre, et le bateau a attendu le bleu.
-papa|Bravo.
 papa|Le quai a eu le temps de se fermer.
 narrateur|Les moufles, sèches, sont rentrées dans le tiroir du banc.
 narrateur|Le bateau sèche contre la patte, face au verre noir.
@@ -17470,7 +17461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17583,6 +17574,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>